<commit_message>
ajout exercice du prof et mise à Kurbenetes
</commit_message>
<xml_diff>
--- a/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
+++ b/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a5f61b3e4cd8107/Inès_perso/M2i_administraeur_CLOUD.0.0/Cours_Python_M2i/KUBERNETES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2393" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B97DE165-EA44-4F40-9E7B-778880EE043B}"/>
+  <xr:revisionPtr revIDLastSave="2409" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AE84D5A-F592-4EA5-B8D9-C35E7E27093E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8D2D9E53-07E4-4E8B-82A4-55704ED06D6A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Listes_des_commandes" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Listes_des_commandes!$A$1:$C$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Listes_des_commandes!$A$1:$C$286</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="624">
   <si>
     <t>Commandes</t>
   </si>
@@ -4702,6 +4702,93 @@
   </si>
   <si>
     <t>Demander au conteneur son nom d'hôte :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Céer un service </t>
+  </si>
+  <si>
+    <t>kubectl expose deployment storefront -n practice-observe --port=80</t>
+  </si>
+  <si>
+    <t>kubectl expose deployment storefront \
+  --name=storefront \
+  --port=80 \
+  --type=ClusterIP \
+  -n practice-observe</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Version encore plus explicite avec un type de Service :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>deployment storefront :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ressource à exposer ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>--port=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">80 : port du Service ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">-n practice-observe : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>espace de noms utilisé.</t>
+    </r>
+  </si>
+  <si>
+    <t>Cette commande crée un Service nommé storefront à partir du Deployment</t>
   </si>
 </sst>
 </file>
@@ -4851,7 +4938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4938,16 +5025,28 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4959,10 +5058,19 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4971,28 +5079,10 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5338,7 +5428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7416C5AA-AA6E-41AB-BBA6-B527D527C8A0}">
-  <dimension ref="A1:C290"/>
+  <dimension ref="A1:C292"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" style="5" bestFit="1" customWidth="1"/>
@@ -5370,7 +5460,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="43" t="s">
         <v>174</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -5381,7 +5471,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="35"/>
+      <c r="A4" s="45"/>
       <c r="B4" s="7" t="s">
         <v>358</v>
       </c>
@@ -5390,2791 +5480,2812 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="9" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="40" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
+        <v>619</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="45"/>
+      <c r="B7" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
-      <c r="B7" s="9" t="s">
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="36"/>
+      <c r="B9" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
-      <c r="B8" s="9" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="36"/>
+      <c r="B10" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C10" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
-      <c r="B9" s="9" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="36"/>
+      <c r="B11" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C11" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
-      <c r="B10" s="9" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="36"/>
+      <c r="B12" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="40"/>
-      <c r="B11" s="9" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="36"/>
+      <c r="B13" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C13" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="40"/>
-      <c r="B12" s="9" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="36"/>
+      <c r="B14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C14" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
-      <c r="B13" s="9" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="36"/>
+      <c r="B15" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
-      <c r="B14" s="9" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="36"/>
+      <c r="B16" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C16" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="39" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="39" t="s">
         <v>187</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
-      <c r="B16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
-      <c r="B17" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="39"/>
       <c r="B18" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C18" s="32"/>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="39"/>
       <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="39"/>
       <c r="B20" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="38"/>
+    </row>
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="39"/>
+      <c r="B21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="39"/>
+      <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="s">
+    <row r="23" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A23" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C23" s="9" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="40"/>
-      <c r="B22" s="9" t="s">
+    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="36"/>
+      <c r="B24" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C24" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
-      <c r="B23" s="9" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="36"/>
+      <c r="B25" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C25" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
-      <c r="B24" s="9" t="s">
+    <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="36"/>
+      <c r="B26" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C26" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
-      <c r="B25" s="9" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="36"/>
+      <c r="B27" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C27" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="39" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="39" t="s">
         <v>188</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
-      <c r="B27" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
-      <c r="B28" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="39"/>
       <c r="B29" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="39"/>
+      <c r="B30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="39"/>
+      <c r="B31" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="36" t="s">
+    <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B32" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="37"/>
-      <c r="B31" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="37"/>
-      <c r="B32" s="9" t="s">
-        <v>86</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="37"/>
+      <c r="A33" s="41"/>
       <c r="B33" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="41"/>
+      <c r="B34" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="41"/>
+      <c r="B35" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C35" s="9" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="37"/>
-      <c r="B34" s="9" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="41"/>
+      <c r="B36" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C36" s="9" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A35" s="37"/>
-      <c r="B35" s="9" t="s">
+    <row r="37" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A37" s="41"/>
+      <c r="B37" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C37" s="9" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="37"/>
-      <c r="B36" s="9" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="41"/>
+      <c r="B38" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="37"/>
-      <c r="B37" s="9" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="41"/>
+      <c r="B39" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="9"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="37"/>
-      <c r="B38" s="9" t="s">
+      <c r="C39" s="9"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="41"/>
+      <c r="B40" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C40" s="9" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="37"/>
-      <c r="B39" s="9" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="41"/>
+      <c r="B41" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C41" s="9" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="37"/>
-      <c r="B40" s="9" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="41"/>
+      <c r="B42" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="37"/>
-      <c r="B41" s="9" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="41"/>
+      <c r="B43" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C43" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="37"/>
-      <c r="B42" s="9" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="41"/>
+      <c r="B44" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C44" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A43" s="37"/>
-      <c r="B43" s="9" t="s">
+    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A45" s="41"/>
+      <c r="B45" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C43" s="30" t="s">
+      <c r="C45" s="30" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A44" s="37"/>
-      <c r="B44" s="9" t="s">
+    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="41"/>
+      <c r="B46" s="9" t="s">
         <v>571</v>
       </c>
-      <c r="C44" s="30" t="s">
+      <c r="C46" s="30" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A45" s="37"/>
-      <c r="B45" s="9" t="s">
+    <row r="47" spans="1:3" ht="210" x14ac:dyDescent="0.25">
+      <c r="A47" s="41"/>
+      <c r="B47" s="9" t="s">
         <v>589</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C47" s="30" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A46" s="37"/>
-      <c r="B46" s="9" t="s">
+    <row r="48" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="41"/>
+      <c r="B48" s="9" t="s">
         <v>591</v>
       </c>
-      <c r="C46" s="30" t="s">
+      <c r="C48" s="30" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="37"/>
-      <c r="B47" s="9" t="s">
+    <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="41"/>
+      <c r="B49" s="9" t="s">
         <v>592</v>
       </c>
-      <c r="C47" s="30" t="s">
+      <c r="C49" s="30" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="38"/>
-      <c r="B48" s="9" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="42"/>
+      <c r="B50" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C50" s="9" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A49" s="39" t="s">
+    <row r="51" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+      <c r="A51" s="39" t="s">
         <v>198</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C51" s="1" t="s">
         <v>597</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="39"/>
-      <c r="B50" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="39"/>
-      <c r="B51" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="39"/>
       <c r="B52" s="1" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="39"/>
       <c r="B53" s="1" t="s">
-        <v>18</v>
+        <v>98</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="39"/>
       <c r="B54" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="39"/>
+      <c r="B55" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A56" s="39"/>
+      <c r="B56" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C56" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="40" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="36" t="s">
         <v>199</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B57" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C57" s="9" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="40"/>
-      <c r="B56" s="9" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="36"/>
+      <c r="B58" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C58" s="9" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="40"/>
-      <c r="B57" s="9" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="36"/>
+      <c r="B59" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C59" s="9" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="40"/>
-      <c r="B58" s="9" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="36"/>
+      <c r="B60" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C60" s="9" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A59" s="39" t="s">
+    <row r="61" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A61" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C61" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
-      <c r="B60" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A61" s="39"/>
-      <c r="B61" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="39"/>
       <c r="B62" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A63" s="39"/>
       <c r="B63" s="1" t="s">
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="39"/>
       <c r="B64" s="1" t="s">
-        <v>148</v>
+        <v>26</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="39"/>
       <c r="B65" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="39"/>
+      <c r="B66" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A67" s="39"/>
+      <c r="B67" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C67" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="40" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="36" t="s">
         <v>203</v>
       </c>
-      <c r="B66" s="9" t="s">
+      <c r="B68" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C68" s="9" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="40"/>
-      <c r="B67" s="9" t="s">
+    <row r="69" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="36"/>
+      <c r="B69" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C69" s="9" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="39" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="39" t="s">
         <v>204</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B70" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C70" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="39"/>
-      <c r="B69" s="1" t="s">
+    <row r="71" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="39"/>
+      <c r="B71" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="40" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="36" t="s">
         <v>205</v>
       </c>
-      <c r="B70" s="9" t="s">
+      <c r="B72" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C72" s="9" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" s="40"/>
-      <c r="B71" s="9" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="36"/>
+      <c r="B73" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C73" s="9" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="40"/>
-      <c r="B72" s="9" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="36"/>
+      <c r="B74" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C74" s="9" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A73" s="40"/>
-      <c r="B73" s="9" t="s">
+    <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A75" s="36"/>
+      <c r="B75" s="9" t="s">
         <v>615</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C75" s="9" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="40"/>
-      <c r="B74" s="9" t="s">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="36"/>
+      <c r="B76" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C76" s="9" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="39" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B77" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C77" s="1" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="39"/>
-      <c r="B76" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" s="39"/>
-      <c r="B77" s="1" t="s">
-        <v>617</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="39"/>
       <c r="B78" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="39"/>
+      <c r="B79" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="39"/>
+      <c r="B80" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C80" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="40" t="s">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="36" t="s">
         <v>207</v>
       </c>
-      <c r="B79" s="9" t="s">
+      <c r="B81" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C81" s="9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" s="40"/>
-      <c r="B80" s="9" t="s">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="36"/>
+      <c r="B82" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C80" s="9" t="s">
+      <c r="C82" s="9" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A81" s="13" t="s">
+    <row r="83" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A83" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B83" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C81" s="1"/>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="36" t="s">
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="40" t="s">
         <v>215</v>
       </c>
-      <c r="B82" s="9" t="s">
+      <c r="B84" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="C82" s="41" t="s">
+      <c r="C84" s="48" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83" s="38"/>
-      <c r="B83" s="9" t="s">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="42"/>
+      <c r="B85" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C83" s="42"/>
-    </row>
-    <row r="84" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="33" t="s">
+      <c r="C85" s="49"/>
+    </row>
+    <row r="86" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="43" t="s">
         <v>219</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B86" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C84" s="6" t="s">
+      <c r="C86" s="6" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="34"/>
-      <c r="B85" s="1" t="s">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="44"/>
+      <c r="B87" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C87" s="6" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" s="34"/>
-      <c r="B86" s="1" t="s">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="44"/>
+      <c r="B88" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C86" s="6" t="s">
+      <c r="C88" s="6" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A87" s="35"/>
-      <c r="B87" s="1" t="s">
+    <row r="89" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A89" s="45"/>
+      <c r="B89" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C87" s="6" t="s">
+      <c r="C89" s="6" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A88" s="14" t="s">
+    <row r="90" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A90" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="B88" s="9" t="s">
+      <c r="B90" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="C88" s="15" t="s">
+      <c r="C90" s="15" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" s="33" t="s">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="43" t="s">
         <v>228</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B91" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="C89" s="6" t="s">
+      <c r="C91" s="6" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" s="35"/>
-      <c r="B90" s="1" t="s">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="45"/>
+      <c r="B92" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="C90" s="6" t="s">
+      <c r="C92" s="6" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="36" t="s">
+    <row r="93" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="40" t="s">
         <v>233</v>
       </c>
-      <c r="B91" s="9" t="s">
+      <c r="B93" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="C91" s="15" t="s">
+      <c r="C93" s="15" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A92" s="38"/>
-      <c r="B92" s="9" t="s">
+    <row r="94" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A94" s="42"/>
+      <c r="B94" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="C92" s="15" t="s">
+      <c r="C94" s="15" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="33" t="s">
+    <row r="95" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="43" t="s">
         <v>234</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B95" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C93" s="6" t="s">
+      <c r="C95" s="6" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A94" s="35"/>
-      <c r="B94" s="1" t="s">
+    <row r="96" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A96" s="45"/>
+      <c r="B96" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="C94" s="6" t="s">
+      <c r="C96" s="6" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="36" t="s">
+    <row r="97" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="40" t="s">
         <v>239</v>
       </c>
-      <c r="B95" s="9" t="s">
+      <c r="B97" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="C95" s="15" t="s">
+      <c r="C97" s="15" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A96" s="37"/>
-      <c r="B96" s="9" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="41"/>
+      <c r="B98" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="C96" s="15" t="s">
+      <c r="C98" s="15" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A97" s="38"/>
-      <c r="B97" s="9" t="s">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="42"/>
+      <c r="B99" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="C97" s="15" t="s">
+      <c r="C99" s="15" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98" s="48" t="s">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="50" t="s">
         <v>246</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B100" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C98" s="6" t="s">
+      <c r="C100" s="6" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="270" x14ac:dyDescent="0.25">
-      <c r="A99" s="49"/>
-      <c r="B99" s="1" t="s">
+    <row r="101" spans="1:3" ht="270" x14ac:dyDescent="0.25">
+      <c r="A101" s="51"/>
+      <c r="B101" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="C99" s="6" t="s">
+      <c r="C101" s="6" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="36" t="s">
+    <row r="102" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="40" t="s">
         <v>261</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="B102" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="C100" s="23" t="s">
+      <c r="C102" s="23" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A101" s="37"/>
-      <c r="B101" s="9" t="s">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="41"/>
+      <c r="B103" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="C101" s="15" t="s">
+      <c r="C103" s="15" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A102" s="37"/>
-      <c r="B102" s="9" t="s">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="41"/>
+      <c r="B104" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="C102" s="15" t="s">
+      <c r="C104" s="15" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" s="37"/>
-      <c r="B103" s="9" t="s">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="41"/>
+      <c r="B105" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="C103" s="15" t="s">
+      <c r="C105" s="15" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" s="38"/>
-      <c r="B104" s="9" t="s">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="42"/>
+      <c r="B106" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="C104" s="15" t="s">
+      <c r="C106" s="15" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="33" t="s">
+    <row r="107" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="43" t="s">
         <v>262</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B107" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C105" s="6" t="s">
+      <c r="C107" s="6" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106" s="34"/>
-      <c r="B106" s="1" t="s">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="44"/>
+      <c r="B108" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="C106" s="6" t="s">
+      <c r="C108" s="6" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" s="35"/>
-      <c r="B107" s="1" t="s">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="45"/>
+      <c r="B109" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="C107" s="6" t="s">
+      <c r="C109" s="6" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="36" t="s">
+    <row r="110" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="40" t="s">
         <v>279</v>
       </c>
-      <c r="B108" s="9" t="s">
+      <c r="B110" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="C108" s="15" t="s">
+      <c r="C110" s="15" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109" s="37"/>
-      <c r="B109" s="9" t="s">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="41"/>
+      <c r="B111" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="C109" s="15" t="s">
+      <c r="C111" s="15" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A110" s="37"/>
-      <c r="B110" s="9" t="s">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="41"/>
+      <c r="B112" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="C110" s="15" t="s">
+      <c r="C112" s="15" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A111" s="37"/>
-      <c r="B111" s="9" t="s">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="41"/>
+      <c r="B113" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="C111" s="15" t="s">
+      <c r="C113" s="15" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A112" s="38"/>
-      <c r="B112" s="9" t="s">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="42"/>
+      <c r="B114" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="C112" s="15" t="s">
+      <c r="C114" s="15" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="33" t="s">
+    <row r="115" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="43" t="s">
         <v>280</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B115" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="C113" s="6" t="s">
+      <c r="C115" s="6" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="35"/>
-      <c r="B114" s="1" t="s">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" s="45"/>
+      <c r="B116" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="C114" s="6" t="s">
+      <c r="C116" s="6" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A115" s="36" t="s">
+    <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A117" s="40" t="s">
         <v>285</v>
       </c>
-      <c r="B115" s="9" t="s">
+      <c r="B117" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="C115" s="15" t="s">
+      <c r="C117" s="15" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A116" s="37"/>
-      <c r="B116" s="9" t="s">
+    <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A118" s="41"/>
+      <c r="B118" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="C116" s="15" t="s">
+      <c r="C118" s="15" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A117" s="38"/>
-      <c r="B117" s="9" t="s">
+    <row r="119" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A119" s="42"/>
+      <c r="B119" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="C117" s="15" t="s">
+      <c r="C119" s="15" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="33" t="s">
+    <row r="120" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="43" t="s">
         <v>292</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B120" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="C118" s="6" t="s">
+      <c r="C120" s="6" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A119" s="34"/>
-      <c r="B119" s="1" t="s">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" s="44"/>
+      <c r="B121" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="C119" s="19" t="s">
+      <c r="C121" s="19" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A120" s="34"/>
-      <c r="B120" s="1" t="s">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" s="44"/>
+      <c r="B122" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C120" s="19" t="s">
+      <c r="C122" s="19" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121" s="35"/>
-      <c r="B121" s="1" t="s">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" s="45"/>
+      <c r="B123" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="C121" s="7" t="s">
+      <c r="C123" s="7" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="36" t="s">
+    <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="40" t="s">
         <v>301</v>
       </c>
-      <c r="B122" s="9" t="s">
+      <c r="B124" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="C122" s="23" t="s">
+      <c r="C124" s="23" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A123" s="38"/>
-      <c r="B123" s="9" t="s">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" s="42"/>
+      <c r="B125" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="C123" s="15" t="s">
+      <c r="C125" s="15" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="33" t="s">
+    <row r="126" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="43" t="s">
         <v>306</v>
       </c>
-      <c r="B124" s="1" t="s">
+      <c r="B126" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C124" s="19" t="s">
+      <c r="C126" s="19" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A125" s="34"/>
-      <c r="B125" s="1" t="s">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" s="44"/>
+      <c r="B127" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="C125" s="19" t="s">
+      <c r="C127" s="19" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A126" s="35"/>
-      <c r="B126" s="1" t="s">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" s="45"/>
+      <c r="B128" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="C126" s="19" t="s">
+      <c r="C128" s="19" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="36" t="s">
+    <row r="129" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="40" t="s">
         <v>312</v>
       </c>
-      <c r="B127" s="9" t="s">
+      <c r="B129" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="C127" s="23" t="s">
+      <c r="C129" s="23" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A128" s="38"/>
-      <c r="B128" s="9" t="s">
+    <row r="130" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A130" s="42"/>
+      <c r="B130" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="C128" s="23"/>
-    </row>
-    <row r="129" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A129" s="16" t="s">
+      <c r="C130" s="23"/>
+    </row>
+    <row r="131" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A131" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="B129" s="17" t="s">
+      <c r="B131" s="17" t="s">
         <v>318</v>
       </c>
-      <c r="C129" s="19" t="s">
+      <c r="C131" s="19" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="36" t="s">
+    <row r="132" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="40" t="s">
         <v>319</v>
       </c>
-      <c r="B130" s="9" t="s">
+      <c r="B132" s="9" t="s">
         <v>320</v>
       </c>
-      <c r="C130" s="23" t="s">
+      <c r="C132" s="23" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A131" s="37"/>
-      <c r="B131" s="8" t="s">
+    <row r="133" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A133" s="41"/>
+      <c r="B133" s="8" t="s">
         <v>323</v>
       </c>
-      <c r="C131" s="23" t="s">
+      <c r="C133" s="23" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A132" s="38"/>
-      <c r="B132" s="9" t="s">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" s="42"/>
+      <c r="B134" s="9" t="s">
         <v>325</v>
       </c>
-      <c r="C132" s="24" t="s">
+      <c r="C134" s="24" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="33" t="s">
+    <row r="135" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="43" t="s">
         <v>326</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B135" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C133" s="19" t="s">
+      <c r="C135" s="19" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" s="35"/>
-      <c r="B134" s="1" t="s">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" s="45"/>
+      <c r="B136" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="C134" s="20" t="s">
+      <c r="C136" s="20" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="36" t="s">
+    <row r="137" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="40" t="s">
         <v>338</v>
       </c>
-      <c r="B135" s="9" t="s">
+      <c r="B137" s="9" t="s">
         <v>331</v>
       </c>
-      <c r="C135" s="9" t="s">
+      <c r="C137" s="9" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A136" s="38"/>
-      <c r="B136" s="9" t="s">
+    <row r="138" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A138" s="42"/>
+      <c r="B138" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="C136" s="23" t="s">
+      <c r="C138" s="23" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="33" t="s">
+    <row r="139" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="43" t="s">
         <v>339</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B139" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="C137" s="19" t="s">
+      <c r="C139" s="19" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A138" s="35"/>
-      <c r="B138" s="1" t="s">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" s="45"/>
+      <c r="B140" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C138" s="19" t="s">
+      <c r="C140" s="19" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A139" s="36" t="s">
+    <row r="141" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A141" s="40" t="s">
         <v>344</v>
       </c>
-      <c r="B139" s="9" t="s">
+      <c r="B141" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="C139" s="23" t="s">
+      <c r="C141" s="23" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="38"/>
-      <c r="B140" s="25" t="s">
+    <row r="142" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="42"/>
+      <c r="B142" s="25" t="s">
         <v>343</v>
       </c>
-      <c r="C140" s="23" t="s">
+      <c r="C142" s="23" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A141" s="16" t="s">
+    <row r="143" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A143" s="16" t="s">
         <v>345</v>
       </c>
-      <c r="B141" s="1" t="s">
+      <c r="B143" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="C141" s="19" t="s">
+      <c r="C143" s="19" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A142" s="36" t="s">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="40" t="s">
         <v>353</v>
       </c>
-      <c r="B142" s="25" t="s">
+      <c r="B144" s="25" t="s">
         <v>331</v>
       </c>
-      <c r="C142" s="23" t="s">
+      <c r="C144" s="23" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A143" s="37"/>
-      <c r="B143" s="9" t="s">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="41"/>
+      <c r="B145" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="C143" s="23" t="s">
+      <c r="C145" s="23" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="38"/>
-      <c r="B144" s="25" t="s">
+    <row r="146" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="42"/>
+      <c r="B146" s="25" t="s">
         <v>352</v>
       </c>
-      <c r="C144" s="23" t="s">
+      <c r="C146" s="23" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="33" t="s">
+    <row r="147" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="43" t="s">
         <v>354</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B147" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C145" s="19" t="s">
+      <c r="C147" s="19" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A146" s="34"/>
-      <c r="B146" s="1" t="s">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="44"/>
+      <c r="B148" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C146" s="19" t="s">
+      <c r="C148" s="19" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147" s="34"/>
-      <c r="B147" s="1" t="s">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="44"/>
+      <c r="B149" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C147" s="19" t="s">
+      <c r="C149" s="19" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="34"/>
-      <c r="B148" s="1" t="s">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="44"/>
+      <c r="B150" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C148" s="19" t="s">
+      <c r="C150" s="19" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" s="35"/>
-      <c r="B149" s="1" t="s">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="45"/>
+      <c r="B151" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C149" s="19"/>
-    </row>
-    <row r="150" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="36" t="s">
+      <c r="C151" s="19"/>
+    </row>
+    <row r="152" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="40" t="s">
         <v>359</v>
       </c>
-      <c r="B150" s="9" t="s">
+      <c r="B152" s="9" t="s">
         <v>361</v>
       </c>
-      <c r="C150" s="23" t="s">
+      <c r="C152" s="23" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151" s="37"/>
-      <c r="B151" s="9" t="s">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="41"/>
+      <c r="B153" s="9" t="s">
         <v>362</v>
       </c>
-      <c r="C151" s="29" t="s">
+      <c r="C153" s="29" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A152" s="37"/>
-      <c r="B152" s="29" t="s">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="41"/>
+      <c r="B154" s="29" t="s">
         <v>365</v>
       </c>
-      <c r="C152" s="23" t="s">
+      <c r="C154" s="23" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153" s="37"/>
-      <c r="B153" s="9" t="s">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="41"/>
+      <c r="B155" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="C153" s="23" t="s">
+      <c r="C155" s="23" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154" s="37"/>
-      <c r="B154" s="9" t="s">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" s="41"/>
+      <c r="B156" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="C154" s="23" t="s">
+      <c r="C156" s="23" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155" s="37"/>
-      <c r="B155" s="9" t="s">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" s="41"/>
+      <c r="B157" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="C155" s="23" t="s">
+      <c r="C157" s="23" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A156" s="38"/>
-      <c r="B156" s="9" t="s">
+    <row r="158" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A158" s="42"/>
+      <c r="B158" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="C156" s="23" t="s">
+      <c r="C158" s="23" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157" s="45" t="s">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="33" t="s">
         <v>374</v>
       </c>
-      <c r="B157" s="21" t="s">
+      <c r="B159" s="21" t="s">
         <v>387</v>
-      </c>
-      <c r="C157" s="21" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A158" s="46"/>
-      <c r="B158" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="C158" s="21" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A159" s="46"/>
-      <c r="B159" s="1" t="s">
-        <v>377</v>
       </c>
       <c r="C159" s="21" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A160" s="46"/>
+      <c r="A160" s="34"/>
       <c r="B160" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C160" s="21" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A161" s="46"/>
+      <c r="A161" s="34"/>
       <c r="B161" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="C161" s="21" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" s="34"/>
+      <c r="B162" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C162" s="21" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" s="34"/>
+      <c r="B163" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="C161" s="19" t="s">
+      <c r="C163" s="19" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A162" s="46"/>
-      <c r="B162" s="1" t="s">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" s="34"/>
+      <c r="B164" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="C162" s="19" t="s">
+      <c r="C164" s="19" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" s="46"/>
-      <c r="B163" s="1" t="s">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" s="34"/>
+      <c r="B165" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="C163" s="20" t="s">
+      <c r="C165" s="20" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A164" s="46"/>
-      <c r="B164" s="1" t="s">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" s="34"/>
+      <c r="B166" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="C164" s="20" t="s">
+      <c r="C166" s="20" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A165" s="47"/>
-      <c r="B165" s="1" t="s">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" s="35"/>
+      <c r="B167" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="C165" s="19" t="s">
+      <c r="C167" s="19" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="36" t="s">
+    <row r="168" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="40" t="s">
         <v>388</v>
       </c>
-      <c r="B166" s="25" t="s">
+      <c r="B168" s="25" t="s">
         <v>390</v>
-      </c>
-      <c r="C166" s="23" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167" s="37"/>
-      <c r="B167" s="9" t="s">
-        <v>391</v>
-      </c>
-      <c r="C167" s="23" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A168" s="37"/>
-      <c r="B168" s="9" t="s">
-        <v>392</v>
       </c>
       <c r="C168" s="23" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169" s="38"/>
+      <c r="A169" s="41"/>
       <c r="B169" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="C169" s="23" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" s="41"/>
+      <c r="B170" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="C170" s="23" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A171" s="42"/>
+      <c r="B171" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="C169" s="23" t="s">
+      <c r="C171" s="23" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A170" s="33" t="s">
+    <row r="172" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="43" t="s">
         <v>395</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B172" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="C170" s="19" t="s">
+      <c r="C172" s="19" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" s="34"/>
-      <c r="B171" s="1" t="s">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" s="44"/>
+      <c r="B173" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="C171" s="19" t="s">
+      <c r="C173" s="19" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A172" s="34"/>
-      <c r="B172" s="1" t="s">
+    <row r="174" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A174" s="44"/>
+      <c r="B174" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="C172" s="19" t="s">
+      <c r="C174" s="19" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173" s="35"/>
-      <c r="B173" s="1" t="s">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" s="45"/>
+      <c r="B175" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="C173" s="19" t="s">
+      <c r="C175" s="19" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A174" s="36" t="s">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" s="40" t="s">
         <v>404</v>
       </c>
-      <c r="B174" s="9" t="s">
+      <c r="B176" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="C174" s="23" t="s">
+      <c r="C176" s="23" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A175" s="37"/>
-      <c r="B175" s="9" t="s">
+    <row r="177" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A177" s="41"/>
+      <c r="B177" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="C175" s="23" t="s">
+      <c r="C177" s="23" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176" s="38"/>
-      <c r="B176" s="9" t="s">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" s="42"/>
+      <c r="B178" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="C176" s="23" t="s">
+      <c r="C178" s="23" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A177" s="33" t="s">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" s="43" t="s">
         <v>410</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B179" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="C177" s="19" t="s">
+      <c r="C179" s="19" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A178" s="34"/>
-      <c r="B178" s="8" t="s">
+    <row r="180" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A180" s="44"/>
+      <c r="B180" s="8" t="s">
         <v>414</v>
       </c>
-      <c r="C178" s="19" t="s">
+      <c r="C180" s="19" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" s="34"/>
-      <c r="B179" s="1" t="s">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" s="44"/>
+      <c r="B181" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="C179" s="19" t="s">
+      <c r="C181" s="19" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A180" s="35"/>
-      <c r="B180" s="1" t="s">
+    <row r="182" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A182" s="45"/>
+      <c r="B182" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="C180" s="19" t="s">
+      <c r="C182" s="19" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="36" t="s">
+    <row r="183" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="40" t="s">
         <v>419</v>
       </c>
-      <c r="B181" s="9" t="s">
+      <c r="B183" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="C181" s="23" t="s">
+      <c r="C183" s="23" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A182" s="37"/>
-      <c r="B182" s="9" t="s">
+    <row r="184" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A184" s="41"/>
+      <c r="B184" s="9" t="s">
         <v>423</v>
       </c>
-      <c r="C182" s="23" t="s">
+      <c r="C184" s="23" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183" s="37"/>
-      <c r="B183" s="9" t="s">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" s="41"/>
+      <c r="B185" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="C183" s="29" t="s">
+      <c r="C185" s="29" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A184" s="38"/>
-      <c r="B184" s="9" t="s">
+    <row r="186" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A186" s="42"/>
+      <c r="B186" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="C184" s="23" t="s">
+      <c r="C186" s="23" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A185" s="33" t="s">
+    <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A187" s="43" t="s">
         <v>428</v>
       </c>
-      <c r="B185" s="1" t="s">
+      <c r="B187" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="C185" s="19" t="s">
+      <c r="C187" s="19" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A186" s="34"/>
-      <c r="B186" s="1" t="s">
+    <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A188" s="44"/>
+      <c r="B188" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="C186" s="19" t="s">
+      <c r="C188" s="19" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A187" s="35"/>
-      <c r="B187" s="1" t="s">
+    <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A189" s="45"/>
+      <c r="B189" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C187" s="19" t="s">
+      <c r="C189" s="19" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A188" s="36" t="s">
+    <row r="190" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="40" t="s">
         <v>435</v>
       </c>
-      <c r="B188" s="9" t="s">
+      <c r="B190" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="C188" s="23" t="s">
+      <c r="C190" s="23" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A189" s="37"/>
-      <c r="B189" s="9" t="s">
+    <row r="191" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A191" s="41"/>
+      <c r="B191" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="C189" s="9" t="s">
+      <c r="C191" s="9" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A190" s="38"/>
-      <c r="B190" s="9" t="s">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" s="42"/>
+      <c r="B192" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="C190" s="23" t="s">
+      <c r="C192" s="23" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A191" s="33" t="s">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" s="43" t="s">
         <v>442</v>
       </c>
-      <c r="B191" s="1" t="s">
+      <c r="B193" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="C191" s="19" t="s">
+      <c r="C193" s="19" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A192" s="34"/>
-      <c r="B192" s="1" t="s">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" s="44"/>
+      <c r="B194" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C192" s="19" t="s">
+      <c r="C194" s="19" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A193" s="34"/>
-      <c r="B193" s="1" t="s">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" s="44"/>
+      <c r="B195" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="C193" s="19" t="s">
+      <c r="C195" s="19" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A194" s="35"/>
-      <c r="B194" s="1" t="s">
+    <row r="196" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A196" s="45"/>
+      <c r="B196" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="C194" s="19" t="s">
+      <c r="C196" s="19" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A195" s="36" t="s">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" s="40" t="s">
         <v>451</v>
       </c>
-      <c r="B195" s="9" t="s">
+      <c r="B197" s="9" t="s">
         <v>390</v>
       </c>
-      <c r="C195" s="23" t="s">
+      <c r="C197" s="23" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A196" s="37"/>
-      <c r="B196" s="9" t="s">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" s="41"/>
+      <c r="B198" s="9" t="s">
         <v>391</v>
       </c>
-      <c r="C196" s="23" t="s">
+      <c r="C198" s="23" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A197" s="37"/>
-      <c r="B197" s="9" t="s">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" s="41"/>
+      <c r="B199" s="9" t="s">
         <v>392</v>
       </c>
-      <c r="C197" s="23" t="s">
+      <c r="C199" s="23" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A198" s="37"/>
-      <c r="B198" s="9" t="s">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" s="41"/>
+      <c r="B200" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="C198" s="23" t="s">
+      <c r="C200" s="23" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A199" s="38"/>
-      <c r="B199" s="9" t="s">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" s="42"/>
+      <c r="B201" s="9" t="s">
         <v>458</v>
       </c>
-      <c r="C199" s="23" t="s">
+      <c r="C201" s="23" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="33" t="s">
+    <row r="202" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="43" t="s">
         <v>459</v>
       </c>
-      <c r="B200" s="1" t="s">
+      <c r="B202" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="C200" s="22" t="s">
+      <c r="C202" s="22" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A201" s="34"/>
-      <c r="B201" s="1" t="s">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" s="44"/>
+      <c r="B203" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="C201" s="22" t="s">
+      <c r="C203" s="22" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A202" s="34"/>
-      <c r="B202" s="1" t="s">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" s="44"/>
+      <c r="B204" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="C202" s="22" t="s">
+      <c r="C204" s="22" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A203" s="35"/>
-      <c r="B203" s="1" t="s">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" s="45"/>
+      <c r="B205" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="C203" s="22" t="s">
+      <c r="C205" s="22" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="204" spans="1:3" ht="270" x14ac:dyDescent="0.25">
-      <c r="A204" s="14" t="s">
+    <row r="206" spans="1:3" ht="270" x14ac:dyDescent="0.25">
+      <c r="A206" s="14" t="s">
         <v>468</v>
       </c>
-      <c r="B204" s="9" t="s">
+      <c r="B206" s="9" t="s">
         <v>489</v>
       </c>
-      <c r="C204" s="23"/>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A205" s="33" t="s">
+      <c r="C206" s="23"/>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" s="43" t="s">
         <v>469</v>
       </c>
-      <c r="B205" s="1" t="s">
+      <c r="B207" s="1" t="s">
         <v>471</v>
-      </c>
-      <c r="C205" s="19" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A206" s="34"/>
-      <c r="B206" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="C206" s="19" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A207" s="34"/>
-      <c r="B207" s="1" t="s">
-        <v>473</v>
       </c>
       <c r="C207" s="19" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A208" s="34"/>
+      <c r="A208" s="44"/>
       <c r="B208" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C208" s="19" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A209" s="44"/>
+      <c r="B209" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C209" s="19" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A210" s="44"/>
+      <c r="B210" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="C208" s="19" t="s">
+      <c r="C210" s="19" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A209" s="34"/>
-      <c r="B209" s="1" t="s">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A211" s="44"/>
+      <c r="B211" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="C209" s="19" t="s">
+      <c r="C211" s="19" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A210" s="34"/>
-      <c r="B210" s="1" t="s">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A212" s="44"/>
+      <c r="B212" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="C210" s="19" t="s">
+      <c r="C212" s="19" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A211" s="34"/>
-      <c r="B211" s="1" t="s">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" s="44"/>
+      <c r="B213" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="C211" s="19" t="s">
+      <c r="C213" s="19" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A212" s="35"/>
-      <c r="B212" s="1" t="s">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A214" s="45"/>
+      <c r="B214" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="C212" s="19" t="s">
+      <c r="C214" s="19" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="213" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A213" s="36" t="s">
+    <row r="215" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="40" t="s">
         <v>482</v>
       </c>
-      <c r="B213" s="9" t="s">
+      <c r="B215" s="9" t="s">
         <v>484</v>
       </c>
-      <c r="C213" s="23" t="s">
+      <c r="C215" s="23" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A214" s="37"/>
-      <c r="B214" s="9" t="s">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A216" s="41"/>
+      <c r="B216" s="9" t="s">
         <v>486</v>
       </c>
-      <c r="C214" s="23" t="s">
+      <c r="C216" s="23" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A215" s="37"/>
-      <c r="B215" s="9" t="s">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" s="41"/>
+      <c r="B217" s="9" t="s">
         <v>487</v>
       </c>
-      <c r="C215" s="23" t="s">
+      <c r="C217" s="23" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A216" s="38"/>
-      <c r="B216" s="9" t="s">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" s="42"/>
+      <c r="B218" s="9" t="s">
         <v>488</v>
       </c>
-      <c r="C216" s="23" t="s">
+      <c r="C218" s="23" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="33" t="s">
+    <row r="219" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="43" t="s">
         <v>527</v>
       </c>
-      <c r="B217" s="1" t="s">
+      <c r="B219" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="C217" s="22" t="s">
+      <c r="C219" s="22" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A218" s="34"/>
-      <c r="B218" s="1" t="s">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" s="44"/>
+      <c r="B220" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="C218" s="28" t="s">
+      <c r="C220" s="28" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A219" s="35"/>
-      <c r="B219" s="1" t="s">
+    <row r="221" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A221" s="45"/>
+      <c r="B221" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="C219" s="22" t="s">
+      <c r="C221" s="22" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="36" t="s">
+    <row r="222" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="40" t="s">
         <v>534</v>
       </c>
-      <c r="B220" s="9" t="s">
+      <c r="B222" s="9" t="s">
         <v>536</v>
       </c>
-      <c r="C220" s="23" t="s">
+      <c r="C222" s="23" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A221" s="37"/>
-      <c r="B221" s="9" t="s">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" s="41"/>
+      <c r="B223" s="9" t="s">
         <v>538</v>
       </c>
-      <c r="C221" s="23" t="s">
+      <c r="C223" s="23" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A222" s="37"/>
-      <c r="B222" s="9" t="s">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" s="41"/>
+      <c r="B224" s="9" t="s">
         <v>540</v>
       </c>
-      <c r="C222" s="23" t="s">
+      <c r="C224" s="23" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A223" s="38"/>
-      <c r="B223" s="9" t="s">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A225" s="42"/>
+      <c r="B225" s="9" t="s">
         <v>542</v>
       </c>
-      <c r="C223" s="23" t="s">
+      <c r="C225" s="23" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A224" s="33" t="s">
+    <row r="226" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="43" t="s">
         <v>543</v>
       </c>
-      <c r="B224" s="1" t="s">
+      <c r="B226" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="C224" s="22" t="s">
+      <c r="C226" s="22" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A225" s="34"/>
-      <c r="B225" s="1" t="s">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A227" s="44"/>
+      <c r="B227" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="C225" s="22" t="s">
+      <c r="C227" s="22" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A226" s="35"/>
-      <c r="B226" s="1" t="s">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A228" s="45"/>
+      <c r="B228" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="C226" s="22" t="s">
+      <c r="C228" s="22" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="36" t="s">
+    <row r="229" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A229" s="40" t="s">
         <v>549</v>
       </c>
-      <c r="B227" s="9" t="s">
+      <c r="B229" s="9" t="s">
         <v>551</v>
       </c>
-      <c r="C227" s="23" t="s">
+      <c r="C229" s="23" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A228" s="37"/>
-      <c r="B228" s="9" t="s">
+    <row r="230" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A230" s="41"/>
+      <c r="B230" s="9" t="s">
         <v>553</v>
       </c>
-      <c r="C228" s="23" t="s">
+      <c r="C230" s="23" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A229" s="38"/>
-      <c r="B229" s="9" t="s">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A231" s="42"/>
+      <c r="B231" s="9" t="s">
         <v>555</v>
       </c>
-      <c r="C229" s="23" t="s">
+      <c r="C231" s="23" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A230" s="33" t="s">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A232" s="43" t="s">
         <v>490</v>
       </c>
-      <c r="B230" s="1" t="s">
+      <c r="B232" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="C230" s="19" t="s">
+      <c r="C232" s="19" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A231" s="34"/>
-      <c r="B231" s="1" t="s">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A233" s="44"/>
+      <c r="B233" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C231" s="19" t="s">
+      <c r="C233" s="19" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A232" s="34"/>
-      <c r="B232" s="1" t="s">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A234" s="44"/>
+      <c r="B234" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="C232" s="19" t="s">
+      <c r="C234" s="19" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A233" s="35"/>
-      <c r="B233" s="1" t="s">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A235" s="45"/>
+      <c r="B235" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="C233" s="19" t="s">
+      <c r="C235" s="19" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="234" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A234" s="14" t="s">
+    <row r="236" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A236" s="14" t="s">
         <v>498</v>
       </c>
-      <c r="B234" s="9" t="s">
+      <c r="B236" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="C234" s="23" t="s">
+      <c r="C236" s="23" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="235" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A235" s="33" t="s">
+    <row r="237" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="43" t="s">
         <v>501</v>
       </c>
-      <c r="B235" s="1" t="s">
+      <c r="B237" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="C235" s="19" t="s">
+      <c r="C237" s="19" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A236" s="34"/>
-      <c r="B236" s="1" t="s">
+    <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A238" s="44"/>
+      <c r="B238" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="C236" s="19" t="s">
+      <c r="C238" s="19" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A237" s="35"/>
-      <c r="B237" s="1" t="s">
+    <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A239" s="45"/>
+      <c r="B239" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="C237" s="19" t="s">
+      <c r="C239" s="19" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A238" s="36" t="s">
+    <row r="240" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A240" s="40" t="s">
         <v>508</v>
       </c>
-      <c r="B238" s="9" t="s">
+      <c r="B240" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="C238" s="23" t="s">
+      <c r="C240" s="23" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A239" s="38"/>
-      <c r="B239" s="9" t="s">
+    <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A241" s="42"/>
+      <c r="B241" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="C239" s="23" t="s">
+      <c r="C241" s="23" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A240" s="33" t="s">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A242" s="43" t="s">
         <v>513</v>
       </c>
-      <c r="B240" s="1" t="s">
+      <c r="B242" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="C240" s="19" t="s">
+      <c r="C242" s="19" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="35"/>
-      <c r="B241" s="1" t="s">
+    <row r="243" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="45"/>
+      <c r="B243" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="C241" s="19" t="s">
+      <c r="C243" s="19" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A242" s="36" t="s">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A244" s="40" t="s">
         <v>518</v>
       </c>
-      <c r="B242" s="9" t="s">
+      <c r="B244" s="9" t="s">
         <v>520</v>
       </c>
-      <c r="C242" s="23" t="s">
+      <c r="C244" s="23" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A243" s="37"/>
-      <c r="B243" s="9" t="s">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A245" s="41"/>
+      <c r="B245" s="9" t="s">
         <v>522</v>
       </c>
-      <c r="C243" s="23" t="s">
+      <c r="C245" s="23" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A244" s="37"/>
-      <c r="B244" s="9" t="s">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A246" s="41"/>
+      <c r="B246" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="C244" s="23" t="s">
+      <c r="C246" s="23" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A245" s="38"/>
-      <c r="B245" s="9" t="s">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A247" s="42"/>
+      <c r="B247" s="9" t="s">
         <v>526</v>
       </c>
-      <c r="C245" s="23" t="s">
+      <c r="C247" s="23" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A246" s="33" t="s">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A248" s="43" t="s">
         <v>556</v>
       </c>
-      <c r="B246" s="1" t="s">
+      <c r="B248" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="C246" s="19" t="s">
+      <c r="C248" s="19" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="247" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A247" s="34"/>
-      <c r="B247" s="1" t="s">
+    <row r="249" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A249" s="44"/>
+      <c r="B249" s="1" t="s">
         <v>560</v>
       </c>
-      <c r="C247" s="19" t="s">
+      <c r="C249" s="19" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A248" s="35"/>
-      <c r="B248" s="1" t="s">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A250" s="45"/>
+      <c r="B250" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="C248" s="19" t="s">
+      <c r="C250" s="19" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="249" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A249" s="36" t="s">
+    <row r="251" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A251" s="40" t="s">
         <v>563</v>
       </c>
-      <c r="B249" s="9" t="s">
+      <c r="B251" s="9" t="s">
         <v>522</v>
       </c>
-      <c r="C249" s="23" t="s">
+      <c r="C251" s="23" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A250" s="37"/>
-      <c r="B250" s="9" t="s">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A252" s="41"/>
+      <c r="B252" s="9" t="s">
         <v>566</v>
       </c>
-      <c r="C250" s="23" t="s">
+      <c r="C252" s="23" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A251" s="37"/>
-      <c r="B251" s="9" t="s">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A253" s="41"/>
+      <c r="B253" s="9" t="s">
         <v>568</v>
       </c>
-      <c r="C251" s="23" t="s">
+      <c r="C253" s="23" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A252" s="38"/>
-      <c r="B252" s="9" t="s">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A254" s="42"/>
+      <c r="B254" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="C252" s="23" t="s">
+      <c r="C254" s="23" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A253" s="16" t="s">
+    <row r="255" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A255" s="16" t="s">
         <v>572</v>
       </c>
-      <c r="B253" s="1" t="s">
+      <c r="B255" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="C253" s="22" t="s">
+      <c r="C255" s="22" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A254" s="33" t="s">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A256" s="43" t="s">
         <v>575</v>
       </c>
-      <c r="B254" s="1" t="s">
+      <c r="B256" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="C254" s="22" t="s">
+      <c r="C256" s="22" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A255" s="34"/>
-      <c r="B255" s="1" t="s">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A257" s="44"/>
+      <c r="B257" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="C255" s="28" t="s">
+      <c r="C257" s="28" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A256" s="34"/>
-      <c r="B256" s="1" t="s">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A258" s="44"/>
+      <c r="B258" s="1" t="s">
         <v>581</v>
       </c>
-      <c r="C256" s="22" t="s">
+      <c r="C258" s="22" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A257" s="35"/>
-      <c r="B257" s="1" t="s">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A259" s="45"/>
+      <c r="B259" s="1" t="s">
         <v>583</v>
       </c>
-      <c r="C257" s="22" t="s">
+      <c r="C259" s="22" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="258" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A258" s="33" t="s">
+    <row r="260" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A260" s="43" t="s">
         <v>584</v>
       </c>
-      <c r="B258" s="1" t="s">
+      <c r="B260" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="C258" s="22" t="s">
+      <c r="C260" s="22" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="259" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A259" s="35"/>
-      <c r="B259" s="1" t="s">
+    <row r="261" spans="1:3" ht="210" x14ac:dyDescent="0.25">
+      <c r="A261" s="45"/>
+      <c r="B261" s="1" t="s">
         <v>588</v>
       </c>
-      <c r="C259" s="22" t="s">
+      <c r="C261" s="22" t="s">
         <v>587</v>
       </c>
-    </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A260" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B260" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="C260" s="1" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A261" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B261" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C261" s="1"/>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="4" t="s">
-        <v>29</v>
+        <v>178</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C262" s="1"/>
-    </row>
-    <row r="263" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+      <c r="C262" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B263" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C263" s="12" t="s">
-        <v>32</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C263" s="1"/>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C264" s="1"/>
     </row>
-    <row r="265" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A265" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B265" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C265" s="1" t="s">
-        <v>39</v>
+        <v>30</v>
+      </c>
+      <c r="B265" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C265" s="12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C266" s="1"/>
+    </row>
+    <row r="267" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A267" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C267" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A268" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B266" s="1" t="s">
+      <c r="B268" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C266" s="1"/>
-    </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A267" s="4" t="s">
+      <c r="C268" s="1"/>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A269" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B267" s="1" t="s">
+      <c r="B269" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C267" s="1"/>
-    </row>
-    <row r="268" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A268" s="4" t="s">
+      <c r="C269" s="1"/>
+    </row>
+    <row r="270" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A270" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="B268" s="1" t="s">
+      <c r="B270" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="C268" s="1" t="s">
+      <c r="C270" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A269" s="31" t="s">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A271" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B269" s="8" t="s">
+      <c r="B271" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C269" s="1"/>
-    </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A270" s="43" t="s">
+      <c r="C271" s="1"/>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A272" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="B270" s="8" t="s">
+      <c r="B272" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C270" s="1"/>
-    </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A271" s="44"/>
-      <c r="B271" s="8" t="s">
+      <c r="C272" s="1"/>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A273" s="47"/>
+      <c r="B273" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C271" s="1"/>
-    </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A272" s="4" t="s">
+      <c r="C273" s="1"/>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A274" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B272" s="1" t="s">
+      <c r="B274" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C272" s="1"/>
-    </row>
-    <row r="273" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A273" s="4" t="s">
+      <c r="C274" s="1"/>
+    </row>
+    <row r="275" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A275" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B273" s="1" t="s">
+      <c r="B275" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C273" s="1" t="s">
+      <c r="C275" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A274" s="39" t="s">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A276" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="B274" s="1" t="s">
+      <c r="B276" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C274" s="1" t="s">
+      <c r="C276" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A275" s="39"/>
-      <c r="B275" s="1" t="s">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A277" s="39"/>
+      <c r="B277" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C275" s="1"/>
-    </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A276" s="39"/>
-      <c r="B276" s="1" t="s">
+      <c r="C277" s="1"/>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" s="39"/>
+      <c r="B278" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C276" s="1"/>
-    </row>
-    <row r="277" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A277" s="4" t="s">
+      <c r="C278" s="1"/>
+    </row>
+    <row r="279" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A279" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B277" s="1" t="s">
+      <c r="B279" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C277" s="1"/>
-    </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A278" s="4" t="s">
+      <c r="C279" s="1"/>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A280" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B278" s="1" t="s">
+      <c r="B280" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C278" s="1"/>
-    </row>
-    <row r="279" spans="1:3" ht="180" x14ac:dyDescent="0.25">
-      <c r="A279" s="33" t="s">
+      <c r="C280" s="1"/>
+    </row>
+    <row r="281" spans="1:3" ht="180" x14ac:dyDescent="0.25">
+      <c r="A281" s="43" t="s">
         <v>600</v>
       </c>
-      <c r="B279" s="1" t="s">
+      <c r="B281" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C279" s="1" t="s">
+      <c r="C281" s="1" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A280" s="34"/>
-      <c r="B280" s="1" t="s">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A282" s="44"/>
+      <c r="B282" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C280" s="32" t="s">
+      <c r="C282" s="38" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A281" s="34"/>
-      <c r="B281" s="1" t="s">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A283" s="44"/>
+      <c r="B283" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C281" s="32"/>
-    </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A282" s="34"/>
-      <c r="B282" s="1" t="s">
+      <c r="C283" s="38"/>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A284" s="44"/>
+      <c r="B284" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C282" s="7" t="s">
+      <c r="C284" s="7" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="A283" s="35"/>
-      <c r="B283" s="1" t="s">
+    <row r="285" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+      <c r="A285" s="45"/>
+      <c r="B285" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="C283" s="1" t="s">
+      <c r="C285" s="1" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="284" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A284" s="4" t="s">
+    <row r="286" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A286" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B284" s="1" t="s">
+      <c r="B286" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C284" s="1" t="s">
+      <c r="C286" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A285" s="45" t="s">
+    <row r="287" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A287" s="33" t="s">
         <v>602</v>
       </c>
-      <c r="B285" s="21" t="s">
+      <c r="B287" s="21" t="s">
         <v>603</v>
       </c>
-      <c r="C285" s="21" t="s">
+      <c r="C287" s="21" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="135" x14ac:dyDescent="0.25">
-      <c r="A286" s="46"/>
-      <c r="B286" s="21" t="s">
+    <row r="288" spans="1:3" ht="135" x14ac:dyDescent="0.25">
+      <c r="A288" s="34"/>
+      <c r="B288" s="21" t="s">
         <v>605</v>
       </c>
-      <c r="C286" s="21" t="s">
+      <c r="C288" s="21" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A287" s="46"/>
-      <c r="B287" s="21" t="s">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A289" s="34"/>
+      <c r="B289" s="21" t="s">
         <v>608</v>
       </c>
-      <c r="C287" s="21" t="s">
+      <c r="C289" s="21" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A288" s="46"/>
-      <c r="B288" s="21" t="s">
+    <row r="290" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A290" s="34"/>
+      <c r="B290" s="21" t="s">
         <v>609</v>
       </c>
-      <c r="C288" s="21" t="s">
+      <c r="C290" s="21" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="289" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A289" s="46"/>
-      <c r="B289" s="21" t="s">
+    <row r="291" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A291" s="34"/>
+      <c r="B291" s="21" t="s">
         <v>610</v>
       </c>
-      <c r="C289" s="21" t="s">
+      <c r="C291" s="21" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A290" s="47"/>
-      <c r="B290" s="21" t="s">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A292" s="35"/>
+      <c r="B292" s="21" t="s">
         <v>614</v>
       </c>
-      <c r="C290" s="21" t="s">
+      <c r="C292" s="21" t="s">
         <v>613</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C284" xr:uid="{7416C5AA-AA6E-41AB-BBA6-B527D527C8A0}"/>
-  <mergeCells count="71">
-    <mergeCell ref="A285:A290"/>
-    <mergeCell ref="A6:A14"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="A79:A80"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A48"/>
-    <mergeCell ref="A157:A165"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A274:A276"/>
-    <mergeCell ref="A246:A248"/>
-    <mergeCell ref="A230:A233"/>
-    <mergeCell ref="A235:A237"/>
-    <mergeCell ref="A238:A239"/>
-    <mergeCell ref="A240:A241"/>
-    <mergeCell ref="A242:A245"/>
-    <mergeCell ref="A191:A194"/>
-    <mergeCell ref="A195:A199"/>
-    <mergeCell ref="A200:A203"/>
-    <mergeCell ref="A205:A212"/>
-    <mergeCell ref="A270:A271"/>
-    <mergeCell ref="A254:A257"/>
-    <mergeCell ref="A258:A259"/>
-    <mergeCell ref="A145:A149"/>
-    <mergeCell ref="A213:A216"/>
-    <mergeCell ref="A174:A176"/>
-    <mergeCell ref="A177:A180"/>
-    <mergeCell ref="A181:A184"/>
-    <mergeCell ref="A185:A187"/>
-    <mergeCell ref="A188:A190"/>
-    <mergeCell ref="A249:A252"/>
-    <mergeCell ref="A217:A219"/>
-    <mergeCell ref="A220:A223"/>
-    <mergeCell ref="A224:A226"/>
-    <mergeCell ref="A227:A229"/>
-    <mergeCell ref="A150:A156"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="A84:A87"/>
-    <mergeCell ref="A89:A90"/>
-    <mergeCell ref="A91:A92"/>
-    <mergeCell ref="A100:A104"/>
-    <mergeCell ref="A93:A94"/>
-    <mergeCell ref="A98:A99"/>
-    <mergeCell ref="A127:A128"/>
-    <mergeCell ref="A113:A114"/>
-    <mergeCell ref="A115:A117"/>
-    <mergeCell ref="A105:A107"/>
-    <mergeCell ref="A108:A112"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="A122:A123"/>
-    <mergeCell ref="A124:A126"/>
-    <mergeCell ref="A82:A83"/>
-    <mergeCell ref="C280:C281"/>
-    <mergeCell ref="A279:A283"/>
+  <autoFilter ref="A1:C286" xr:uid="{7416C5AA-AA6E-41AB-BBA6-B527D527C8A0}"/>
+  <mergeCells count="72">
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="C282:C283"/>
+    <mergeCell ref="A281:A285"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A142:A144"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="A133:A134"/>
+    <mergeCell ref="A144:A146"/>
+    <mergeCell ref="A132:A134"/>
     <mergeCell ref="A135:A136"/>
     <mergeCell ref="A137:A138"/>
     <mergeCell ref="A139:A140"/>
-    <mergeCell ref="A15:A20"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A59:A65"/>
-    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="A141:A142"/>
+    <mergeCell ref="A17:A22"/>
+    <mergeCell ref="A51:A56"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="A61:A67"/>
     <mergeCell ref="A68:A69"/>
-    <mergeCell ref="A70:A74"/>
+    <mergeCell ref="A70:A71"/>
+    <mergeCell ref="A72:A76"/>
+    <mergeCell ref="A77:A80"/>
+    <mergeCell ref="A97:A99"/>
+    <mergeCell ref="A120:A123"/>
+    <mergeCell ref="A124:A125"/>
+    <mergeCell ref="A126:A128"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A114"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="A102:A106"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="A100:A101"/>
+    <mergeCell ref="A272:A273"/>
+    <mergeCell ref="A256:A259"/>
+    <mergeCell ref="A260:A261"/>
+    <mergeCell ref="A147:A151"/>
+    <mergeCell ref="A215:A218"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A182"/>
+    <mergeCell ref="A183:A186"/>
+    <mergeCell ref="A187:A189"/>
+    <mergeCell ref="A190:A192"/>
+    <mergeCell ref="A251:A254"/>
+    <mergeCell ref="A219:A221"/>
+    <mergeCell ref="A222:A225"/>
+    <mergeCell ref="A226:A228"/>
+    <mergeCell ref="A229:A231"/>
+    <mergeCell ref="A152:A158"/>
+    <mergeCell ref="A244:A247"/>
+    <mergeCell ref="A193:A196"/>
+    <mergeCell ref="A197:A201"/>
+    <mergeCell ref="A202:A205"/>
+    <mergeCell ref="A207:A214"/>
+    <mergeCell ref="A287:A292"/>
+    <mergeCell ref="A8:A16"/>
+    <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A32:A50"/>
+    <mergeCell ref="A159:A167"/>
+    <mergeCell ref="A168:A171"/>
+    <mergeCell ref="A172:A175"/>
+    <mergeCell ref="A276:A278"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A232:A235"/>
+    <mergeCell ref="A237:A239"/>
+    <mergeCell ref="A240:A241"/>
+    <mergeCell ref="A242:A243"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
mise à jour kubernetes
</commit_message>
<xml_diff>
--- a/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
+++ b/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a5f61b3e4cd8107/Inès_perso/M2i_administraeur_CLOUD.0.0/Cours_Python_M2i/KUBERNETES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2409" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AE84D5A-F592-4EA5-B8D9-C35E7E27093E}"/>
+  <xr:revisionPtr revIDLastSave="2410" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{334E8C58-A663-4A65-B402-4BE34D0BDBD7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8D2D9E53-07E4-4E8B-82A4-55704ED06D6A}"/>
   </bookViews>
@@ -5028,25 +5028,16 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5058,19 +5049,10 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5083,6 +5065,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5460,7 +5460,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="33" t="s">
         <v>174</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -5471,7 +5471,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="45"/>
+      <c r="A4" s="34"/>
       <c r="B4" s="7" t="s">
         <v>358</v>
       </c>
@@ -5491,7 +5491,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="44" t="s">
         <v>619</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -5511,7 +5511,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="41" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="9" t="s">
@@ -5522,7 +5522,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
+      <c r="A9" s="41"/>
       <c r="B9" s="9" t="s">
         <v>172</v>
       </c>
@@ -5531,7 +5531,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="36"/>
+      <c r="A10" s="41"/>
       <c r="B10" s="9" t="s">
         <v>54</v>
       </c>
@@ -5540,7 +5540,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="36"/>
+      <c r="A11" s="41"/>
       <c r="B11" s="9" t="s">
         <v>56</v>
       </c>
@@ -5549,7 +5549,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="36"/>
+      <c r="A12" s="41"/>
       <c r="B12" s="9" t="s">
         <v>58</v>
       </c>
@@ -5558,7 +5558,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
+      <c r="A13" s="41"/>
       <c r="B13" s="9" t="s">
         <v>59</v>
       </c>
@@ -5567,7 +5567,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="36"/>
+      <c r="A14" s="41"/>
       <c r="B14" s="9" t="s">
         <v>62</v>
       </c>
@@ -5576,7 +5576,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="36"/>
+      <c r="A15" s="41"/>
       <c r="B15" s="9" t="s">
         <v>10</v>
       </c>
@@ -5585,7 +5585,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="36"/>
+      <c r="A16" s="41"/>
       <c r="B16" s="9" t="s">
         <v>4</v>
       </c>
@@ -5594,7 +5594,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="40" t="s">
         <v>187</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -5605,7 +5605,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="1" t="s">
         <v>6</v>
       </c>
@@ -5614,23 +5614,23 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="35" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="38"/>
+      <c r="C20" s="35"/>
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="40"/>
       <c r="B21" s="1" t="s">
         <v>17</v>
       </c>
@@ -5639,7 +5639,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="40"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -5648,7 +5648,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="51" t="s">
         <v>77</v>
       </c>
       <c r="B23" s="9" t="s">
@@ -5659,7 +5659,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="36"/>
+      <c r="A24" s="41"/>
       <c r="B24" s="9" t="s">
         <v>8</v>
       </c>
@@ -5668,7 +5668,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="36"/>
+      <c r="A25" s="41"/>
       <c r="B25" s="9" t="s">
         <v>68</v>
       </c>
@@ -5677,7 +5677,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="36"/>
+      <c r="A26" s="41"/>
       <c r="B26" s="9" t="s">
         <v>22</v>
       </c>
@@ -5686,7 +5686,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
+      <c r="A27" s="41"/>
       <c r="B27" s="9" t="s">
         <v>69</v>
       </c>
@@ -5695,7 +5695,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="40" t="s">
         <v>188</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -5706,7 +5706,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="1" t="s">
         <v>212</v>
       </c>
@@ -5715,7 +5715,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="1" t="s">
         <v>84</v>
       </c>
@@ -5724,7 +5724,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="40"/>
       <c r="B31" s="1" t="s">
         <v>144</v>
       </c>
@@ -5733,7 +5733,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="37" t="s">
         <v>197</v>
       </c>
       <c r="B32" s="9" t="s">
@@ -5744,7 +5744,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="41"/>
+      <c r="A33" s="38"/>
       <c r="B33" s="9" t="s">
         <v>190</v>
       </c>
@@ -5753,7 +5753,7 @@
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="41"/>
+      <c r="A34" s="38"/>
       <c r="B34" s="9" t="s">
         <v>86</v>
       </c>
@@ -5762,7 +5762,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="41"/>
+      <c r="A35" s="38"/>
       <c r="B35" s="9" t="s">
         <v>64</v>
       </c>
@@ -5771,7 +5771,7 @@
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="41"/>
+      <c r="A36" s="38"/>
       <c r="B36" s="9" t="s">
         <v>88</v>
       </c>
@@ -5780,7 +5780,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A37" s="41"/>
+      <c r="A37" s="38"/>
       <c r="B37" s="9" t="s">
         <v>20</v>
       </c>
@@ -5789,7 +5789,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="41"/>
+      <c r="A38" s="38"/>
       <c r="B38" s="9" t="s">
         <v>90</v>
       </c>
@@ -5798,14 +5798,14 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="41"/>
+      <c r="A39" s="38"/>
       <c r="B39" s="9" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="9"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="41"/>
+      <c r="A40" s="38"/>
       <c r="B40" s="9" t="s">
         <v>91</v>
       </c>
@@ -5814,7 +5814,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="41"/>
+      <c r="A41" s="38"/>
       <c r="B41" s="9" t="s">
         <v>94</v>
       </c>
@@ -5823,7 +5823,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="41"/>
+      <c r="A42" s="38"/>
       <c r="B42" s="9" t="s">
         <v>92</v>
       </c>
@@ -5832,7 +5832,7 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="41"/>
+      <c r="A43" s="38"/>
       <c r="B43" s="9" t="s">
         <v>14</v>
       </c>
@@ -5841,7 +5841,7 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="41"/>
+      <c r="A44" s="38"/>
       <c r="B44" s="9" t="s">
         <v>15</v>
       </c>
@@ -5850,7 +5850,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A45" s="41"/>
+      <c r="A45" s="38"/>
       <c r="B45" s="9" t="s">
         <v>19</v>
       </c>
@@ -5859,7 +5859,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A46" s="41"/>
+      <c r="A46" s="38"/>
       <c r="B46" s="9" t="s">
         <v>571</v>
       </c>
@@ -5868,7 +5868,7 @@
       </c>
     </row>
     <row r="47" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A47" s="41"/>
+      <c r="A47" s="38"/>
       <c r="B47" s="9" t="s">
         <v>589</v>
       </c>
@@ -5877,7 +5877,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="41"/>
+      <c r="A48" s="38"/>
       <c r="B48" s="9" t="s">
         <v>591</v>
       </c>
@@ -5886,7 +5886,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="41"/>
+      <c r="A49" s="38"/>
       <c r="B49" s="9" t="s">
         <v>592</v>
       </c>
@@ -5895,7 +5895,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="42"/>
+      <c r="A50" s="39"/>
       <c r="B50" s="9" t="s">
         <v>93</v>
       </c>
@@ -5904,7 +5904,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A51" s="39" t="s">
+      <c r="A51" s="40" t="s">
         <v>198</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -5915,7 +5915,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="39"/>
+      <c r="A52" s="40"/>
       <c r="B52" s="1" t="s">
         <v>96</v>
       </c>
@@ -5924,7 +5924,7 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="39"/>
+      <c r="A53" s="40"/>
       <c r="B53" s="1" t="s">
         <v>98</v>
       </c>
@@ -5933,7 +5933,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="39"/>
+      <c r="A54" s="40"/>
       <c r="B54" s="1" t="s">
         <v>71</v>
       </c>
@@ -5942,7 +5942,7 @@
       </c>
     </row>
     <row r="55" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="39"/>
+      <c r="A55" s="40"/>
       <c r="B55" s="1" t="s">
         <v>18</v>
       </c>
@@ -5951,7 +5951,7 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A56" s="39"/>
+      <c r="A56" s="40"/>
       <c r="B56" s="1" t="s">
         <v>99</v>
       </c>
@@ -5960,7 +5960,7 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="36" t="s">
+      <c r="A57" s="41" t="s">
         <v>199</v>
       </c>
       <c r="B57" s="9" t="s">
@@ -5971,7 +5971,7 @@
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="36"/>
+      <c r="A58" s="41"/>
       <c r="B58" s="9" t="s">
         <v>101</v>
       </c>
@@ -5980,7 +5980,7 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="36"/>
+      <c r="A59" s="41"/>
       <c r="B59" s="9" t="s">
         <v>103</v>
       </c>
@@ -5989,7 +5989,7 @@
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="36"/>
+      <c r="A60" s="41"/>
       <c r="B60" s="9" t="s">
         <v>106</v>
       </c>
@@ -5998,7 +5998,7 @@
       </c>
     </row>
     <row r="61" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A61" s="39" t="s">
+      <c r="A61" s="40" t="s">
         <v>200</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -6009,7 +6009,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="39"/>
+      <c r="A62" s="40"/>
       <c r="B62" s="1" t="s">
         <v>107</v>
       </c>
@@ -6018,7 +6018,7 @@
       </c>
     </row>
     <row r="63" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A63" s="39"/>
+      <c r="A63" s="40"/>
       <c r="B63" s="1" t="s">
         <v>110</v>
       </c>
@@ -6027,7 +6027,7 @@
       </c>
     </row>
     <row r="64" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64" s="39"/>
+      <c r="A64" s="40"/>
       <c r="B64" s="1" t="s">
         <v>26</v>
       </c>
@@ -6036,7 +6036,7 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="39"/>
+      <c r="A65" s="40"/>
       <c r="B65" s="1" t="s">
         <v>36</v>
       </c>
@@ -6045,7 +6045,7 @@
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="39"/>
+      <c r="A66" s="40"/>
       <c r="B66" s="1" t="s">
         <v>148</v>
       </c>
@@ -6054,7 +6054,7 @@
       </c>
     </row>
     <row r="67" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A67" s="39"/>
+      <c r="A67" s="40"/>
       <c r="B67" s="1" t="s">
         <v>50</v>
       </c>
@@ -6063,7 +6063,7 @@
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="36" t="s">
+      <c r="A68" s="41" t="s">
         <v>203</v>
       </c>
       <c r="B68" s="9" t="s">
@@ -6074,7 +6074,7 @@
       </c>
     </row>
     <row r="69" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="36"/>
+      <c r="A69" s="41"/>
       <c r="B69" s="9" t="s">
         <v>114</v>
       </c>
@@ -6083,7 +6083,7 @@
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="39" t="s">
+      <c r="A70" s="40" t="s">
         <v>204</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -6094,7 +6094,7 @@
       </c>
     </row>
     <row r="71" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="39"/>
+      <c r="A71" s="40"/>
       <c r="B71" s="1" t="s">
         <v>122</v>
       </c>
@@ -6103,7 +6103,7 @@
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="36" t="s">
+      <c r="A72" s="41" t="s">
         <v>205</v>
       </c>
       <c r="B72" s="9" t="s">
@@ -6114,7 +6114,7 @@
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="36"/>
+      <c r="A73" s="41"/>
       <c r="B73" s="9" t="s">
         <v>126</v>
       </c>
@@ -6123,7 +6123,7 @@
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="36"/>
+      <c r="A74" s="41"/>
       <c r="B74" s="9" t="s">
         <v>128</v>
       </c>
@@ -6132,7 +6132,7 @@
       </c>
     </row>
     <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A75" s="36"/>
+      <c r="A75" s="41"/>
       <c r="B75" s="9" t="s">
         <v>615</v>
       </c>
@@ -6141,7 +6141,7 @@
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="36"/>
+      <c r="A76" s="41"/>
       <c r="B76" s="9" t="s">
         <v>130</v>
       </c>
@@ -6150,7 +6150,7 @@
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" s="39" t="s">
+      <c r="A77" s="40" t="s">
         <v>206</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -6161,7 +6161,7 @@
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="39"/>
+      <c r="A78" s="40"/>
       <c r="B78" s="1" t="s">
         <v>134</v>
       </c>
@@ -6170,7 +6170,7 @@
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="39"/>
+      <c r="A79" s="40"/>
       <c r="B79" s="1" t="s">
         <v>617</v>
       </c>
@@ -6179,7 +6179,7 @@
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" s="39"/>
+      <c r="A80" s="40"/>
       <c r="B80" s="1" t="s">
         <v>136</v>
       </c>
@@ -6188,7 +6188,7 @@
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" s="36" t="s">
+      <c r="A81" s="41" t="s">
         <v>207</v>
       </c>
       <c r="B81" s="9" t="s">
@@ -6199,7 +6199,7 @@
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="36"/>
+      <c r="A82" s="41"/>
       <c r="B82" s="9" t="s">
         <v>139</v>
       </c>
@@ -6217,25 +6217,25 @@
       <c r="C83" s="1"/>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" s="40" t="s">
+      <c r="A84" s="37" t="s">
         <v>215</v>
       </c>
       <c r="B84" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="C84" s="48" t="s">
+      <c r="C84" s="42" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="42"/>
+      <c r="A85" s="39"/>
       <c r="B85" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C85" s="49"/>
+      <c r="C85" s="43"/>
     </row>
     <row r="86" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="43" t="s">
+      <c r="A86" s="33" t="s">
         <v>219</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -6246,7 +6246,7 @@
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="44"/>
+      <c r="A87" s="36"/>
       <c r="B87" s="1" t="s">
         <v>156</v>
       </c>
@@ -6255,7 +6255,7 @@
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" s="44"/>
+      <c r="A88" s="36"/>
       <c r="B88" s="1" t="s">
         <v>157</v>
       </c>
@@ -6264,7 +6264,7 @@
       </c>
     </row>
     <row r="89" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A89" s="45"/>
+      <c r="A89" s="34"/>
       <c r="B89" s="1" t="s">
         <v>220</v>
       </c>
@@ -6284,7 +6284,7 @@
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="43" t="s">
+      <c r="A91" s="33" t="s">
         <v>228</v>
       </c>
       <c r="B91" s="1" t="s">
@@ -6295,7 +6295,7 @@
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" s="45"/>
+      <c r="A92" s="34"/>
       <c r="B92" s="1" t="s">
         <v>227</v>
       </c>
@@ -6304,7 +6304,7 @@
       </c>
     </row>
     <row r="93" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="40" t="s">
+      <c r="A93" s="37" t="s">
         <v>233</v>
       </c>
       <c r="B93" s="9" t="s">
@@ -6315,7 +6315,7 @@
       </c>
     </row>
     <row r="94" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A94" s="42"/>
+      <c r="A94" s="39"/>
       <c r="B94" s="9" t="s">
         <v>232</v>
       </c>
@@ -6324,7 +6324,7 @@
       </c>
     </row>
     <row r="95" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="43" t="s">
+      <c r="A95" s="33" t="s">
         <v>234</v>
       </c>
       <c r="B95" s="1" t="s">
@@ -6335,7 +6335,7 @@
       </c>
     </row>
     <row r="96" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A96" s="45"/>
+      <c r="A96" s="34"/>
       <c r="B96" s="1" t="s">
         <v>237</v>
       </c>
@@ -6344,7 +6344,7 @@
       </c>
     </row>
     <row r="97" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="40" t="s">
+      <c r="A97" s="37" t="s">
         <v>239</v>
       </c>
       <c r="B97" s="9" t="s">
@@ -6355,7 +6355,7 @@
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98" s="41"/>
+      <c r="A98" s="38"/>
       <c r="B98" s="9" t="s">
         <v>243</v>
       </c>
@@ -6364,7 +6364,7 @@
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A99" s="42"/>
+      <c r="A99" s="39"/>
       <c r="B99" s="9" t="s">
         <v>245</v>
       </c>
@@ -6373,7 +6373,7 @@
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A100" s="50" t="s">
+      <c r="A100" s="44" t="s">
         <v>246</v>
       </c>
       <c r="B100" s="1" t="s">
@@ -6384,7 +6384,7 @@
       </c>
     </row>
     <row r="101" spans="1:3" ht="270" x14ac:dyDescent="0.25">
-      <c r="A101" s="51"/>
+      <c r="A101" s="45"/>
       <c r="B101" s="1" t="s">
         <v>250</v>
       </c>
@@ -6393,7 +6393,7 @@
       </c>
     </row>
     <row r="102" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="40" t="s">
+      <c r="A102" s="37" t="s">
         <v>261</v>
       </c>
       <c r="B102" s="9" t="s">
@@ -6404,7 +6404,7 @@
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" s="41"/>
+      <c r="A103" s="38"/>
       <c r="B103" s="9" t="s">
         <v>254</v>
       </c>
@@ -6413,7 +6413,7 @@
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" s="41"/>
+      <c r="A104" s="38"/>
       <c r="B104" s="9" t="s">
         <v>256</v>
       </c>
@@ -6422,7 +6422,7 @@
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A105" s="41"/>
+      <c r="A105" s="38"/>
       <c r="B105" s="9" t="s">
         <v>257</v>
       </c>
@@ -6431,7 +6431,7 @@
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106" s="42"/>
+      <c r="A106" s="39"/>
       <c r="B106" s="9" t="s">
         <v>260</v>
       </c>
@@ -6440,7 +6440,7 @@
       </c>
     </row>
     <row r="107" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="43" t="s">
+      <c r="A107" s="33" t="s">
         <v>262</v>
       </c>
       <c r="B107" s="1" t="s">
@@ -6451,7 +6451,7 @@
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A108" s="44"/>
+      <c r="A108" s="36"/>
       <c r="B108" s="1" t="s">
         <v>266</v>
       </c>
@@ -6460,7 +6460,7 @@
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109" s="45"/>
+      <c r="A109" s="34"/>
       <c r="B109" s="1" t="s">
         <v>267</v>
       </c>
@@ -6469,7 +6469,7 @@
       </c>
     </row>
     <row r="110" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="40" t="s">
+      <c r="A110" s="37" t="s">
         <v>279</v>
       </c>
       <c r="B110" s="9" t="s">
@@ -6480,7 +6480,7 @@
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A111" s="41"/>
+      <c r="A111" s="38"/>
       <c r="B111" s="9" t="s">
         <v>272</v>
       </c>
@@ -6489,7 +6489,7 @@
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A112" s="41"/>
+      <c r="A112" s="38"/>
       <c r="B112" s="9" t="s">
         <v>273</v>
       </c>
@@ -6498,7 +6498,7 @@
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A113" s="41"/>
+      <c r="A113" s="38"/>
       <c r="B113" s="9" t="s">
         <v>275</v>
       </c>
@@ -6507,7 +6507,7 @@
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="42"/>
+      <c r="A114" s="39"/>
       <c r="B114" s="9" t="s">
         <v>278</v>
       </c>
@@ -6516,7 +6516,7 @@
       </c>
     </row>
     <row r="115" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="43" t="s">
+      <c r="A115" s="33" t="s">
         <v>280</v>
       </c>
       <c r="B115" s="1" t="s">
@@ -6527,7 +6527,7 @@
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116" s="45"/>
+      <c r="A116" s="34"/>
       <c r="B116" s="1" t="s">
         <v>284</v>
       </c>
@@ -6536,7 +6536,7 @@
       </c>
     </row>
     <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A117" s="40" t="s">
+      <c r="A117" s="37" t="s">
         <v>285</v>
       </c>
       <c r="B117" s="9" t="s">
@@ -6547,7 +6547,7 @@
       </c>
     </row>
     <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A118" s="41"/>
+      <c r="A118" s="38"/>
       <c r="B118" s="9" t="s">
         <v>289</v>
       </c>
@@ -6556,7 +6556,7 @@
       </c>
     </row>
     <row r="119" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A119" s="42"/>
+      <c r="A119" s="39"/>
       <c r="B119" s="9" t="s">
         <v>291</v>
       </c>
@@ -6565,7 +6565,7 @@
       </c>
     </row>
     <row r="120" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="43" t="s">
+      <c r="A120" s="33" t="s">
         <v>292</v>
       </c>
       <c r="B120" s="1" t="s">
@@ -6576,7 +6576,7 @@
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121" s="44"/>
+      <c r="A121" s="36"/>
       <c r="B121" s="1" t="s">
         <v>296</v>
       </c>
@@ -6585,7 +6585,7 @@
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A122" s="44"/>
+      <c r="A122" s="36"/>
       <c r="B122" s="1" t="s">
         <v>298</v>
       </c>
@@ -6594,7 +6594,7 @@
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A123" s="45"/>
+      <c r="A123" s="34"/>
       <c r="B123" s="1" t="s">
         <v>300</v>
       </c>
@@ -6603,7 +6603,7 @@
       </c>
     </row>
     <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="40" t="s">
+      <c r="A124" s="37" t="s">
         <v>301</v>
       </c>
       <c r="B124" s="9" t="s">
@@ -6614,7 +6614,7 @@
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A125" s="42"/>
+      <c r="A125" s="39"/>
       <c r="B125" s="9" t="s">
         <v>305</v>
       </c>
@@ -6623,7 +6623,7 @@
       </c>
     </row>
     <row r="126" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="43" t="s">
+      <c r="A126" s="33" t="s">
         <v>306</v>
       </c>
       <c r="B126" s="1" t="s">
@@ -6634,7 +6634,7 @@
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127" s="44"/>
+      <c r="A127" s="36"/>
       <c r="B127" s="1" t="s">
         <v>309</v>
       </c>
@@ -6643,7 +6643,7 @@
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128" s="45"/>
+      <c r="A128" s="34"/>
       <c r="B128" s="1" t="s">
         <v>311</v>
       </c>
@@ -6652,7 +6652,7 @@
       </c>
     </row>
     <row r="129" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="40" t="s">
+      <c r="A129" s="37" t="s">
         <v>312</v>
       </c>
       <c r="B129" s="9" t="s">
@@ -6663,7 +6663,7 @@
       </c>
     </row>
     <row r="130" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A130" s="42"/>
+      <c r="A130" s="39"/>
       <c r="B130" s="9" t="s">
         <v>315</v>
       </c>
@@ -6681,7 +6681,7 @@
       </c>
     </row>
     <row r="132" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="40" t="s">
+      <c r="A132" s="37" t="s">
         <v>319</v>
       </c>
       <c r="B132" s="9" t="s">
@@ -6692,7 +6692,7 @@
       </c>
     </row>
     <row r="133" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A133" s="41"/>
+      <c r="A133" s="38"/>
       <c r="B133" s="8" t="s">
         <v>323</v>
       </c>
@@ -6701,7 +6701,7 @@
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" s="42"/>
+      <c r="A134" s="39"/>
       <c r="B134" s="9" t="s">
         <v>325</v>
       </c>
@@ -6710,7 +6710,7 @@
       </c>
     </row>
     <row r="135" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="43" t="s">
+      <c r="A135" s="33" t="s">
         <v>326</v>
       </c>
       <c r="B135" s="1" t="s">
@@ -6721,7 +6721,7 @@
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A136" s="45"/>
+      <c r="A136" s="34"/>
       <c r="B136" s="1" t="s">
         <v>330</v>
       </c>
@@ -6730,7 +6730,7 @@
       </c>
     </row>
     <row r="137" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="40" t="s">
+      <c r="A137" s="37" t="s">
         <v>338</v>
       </c>
       <c r="B137" s="9" t="s">
@@ -6741,7 +6741,7 @@
       </c>
     </row>
     <row r="138" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A138" s="42"/>
+      <c r="A138" s="39"/>
       <c r="B138" s="9" t="s">
         <v>334</v>
       </c>
@@ -6750,7 +6750,7 @@
       </c>
     </row>
     <row r="139" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="43" t="s">
+      <c r="A139" s="33" t="s">
         <v>339</v>
       </c>
       <c r="B139" s="1" t="s">
@@ -6761,7 +6761,7 @@
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A140" s="45"/>
+      <c r="A140" s="34"/>
       <c r="B140" s="1" t="s">
         <v>328</v>
       </c>
@@ -6770,7 +6770,7 @@
       </c>
     </row>
     <row r="141" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A141" s="40" t="s">
+      <c r="A141" s="37" t="s">
         <v>344</v>
       </c>
       <c r="B141" s="9" t="s">
@@ -6781,7 +6781,7 @@
       </c>
     </row>
     <row r="142" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="42"/>
+      <c r="A142" s="39"/>
       <c r="B142" s="25" t="s">
         <v>343</v>
       </c>
@@ -6801,7 +6801,7 @@
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A144" s="40" t="s">
+      <c r="A144" s="37" t="s">
         <v>353</v>
       </c>
       <c r="B144" s="25" t="s">
@@ -6812,7 +6812,7 @@
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" s="41"/>
+      <c r="A145" s="38"/>
       <c r="B145" s="9" t="s">
         <v>350</v>
       </c>
@@ -6821,7 +6821,7 @@
       </c>
     </row>
     <row r="146" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="42"/>
+      <c r="A146" s="39"/>
       <c r="B146" s="25" t="s">
         <v>352</v>
       </c>
@@ -6830,7 +6830,7 @@
       </c>
     </row>
     <row r="147" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="43" t="s">
+      <c r="A147" s="33" t="s">
         <v>354</v>
       </c>
       <c r="B147" s="1" t="s">
@@ -6841,7 +6841,7 @@
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="44"/>
+      <c r="A148" s="36"/>
       <c r="B148" s="1" t="s">
         <v>156</v>
       </c>
@@ -6850,7 +6850,7 @@
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" s="44"/>
+      <c r="A149" s="36"/>
       <c r="B149" s="1" t="s">
         <v>157</v>
       </c>
@@ -6859,7 +6859,7 @@
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150" s="44"/>
+      <c r="A150" s="36"/>
       <c r="B150" s="1" t="s">
         <v>159</v>
       </c>
@@ -6868,14 +6868,14 @@
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151" s="45"/>
+      <c r="A151" s="34"/>
       <c r="B151" s="1" t="s">
         <v>160</v>
       </c>
       <c r="C151" s="19"/>
     </row>
     <row r="152" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="40" t="s">
+      <c r="A152" s="37" t="s">
         <v>359</v>
       </c>
       <c r="B152" s="9" t="s">
@@ -6886,7 +6886,7 @@
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153" s="41"/>
+      <c r="A153" s="38"/>
       <c r="B153" s="9" t="s">
         <v>362</v>
       </c>
@@ -6895,7 +6895,7 @@
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154" s="41"/>
+      <c r="A154" s="38"/>
       <c r="B154" s="29" t="s">
         <v>365</v>
       </c>
@@ -6904,7 +6904,7 @@
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155" s="41"/>
+      <c r="A155" s="38"/>
       <c r="B155" s="9" t="s">
         <v>367</v>
       </c>
@@ -6913,7 +6913,7 @@
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A156" s="41"/>
+      <c r="A156" s="38"/>
       <c r="B156" s="9" t="s">
         <v>369</v>
       </c>
@@ -6922,7 +6922,7 @@
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157" s="41"/>
+      <c r="A157" s="38"/>
       <c r="B157" s="9" t="s">
         <v>371</v>
       </c>
@@ -6931,7 +6931,7 @@
       </c>
     </row>
     <row r="158" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A158" s="42"/>
+      <c r="A158" s="39"/>
       <c r="B158" s="9" t="s">
         <v>373</v>
       </c>
@@ -6940,7 +6940,7 @@
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A159" s="33" t="s">
+      <c r="A159" s="48" t="s">
         <v>374</v>
       </c>
       <c r="B159" s="21" t="s">
@@ -6951,7 +6951,7 @@
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A160" s="34"/>
+      <c r="A160" s="49"/>
       <c r="B160" s="1" t="s">
         <v>376</v>
       </c>
@@ -6960,7 +6960,7 @@
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A161" s="34"/>
+      <c r="A161" s="49"/>
       <c r="B161" s="1" t="s">
         <v>377</v>
       </c>
@@ -6969,7 +6969,7 @@
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A162" s="34"/>
+      <c r="A162" s="49"/>
       <c r="B162" s="1" t="s">
         <v>378</v>
       </c>
@@ -6978,7 +6978,7 @@
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" s="34"/>
+      <c r="A163" s="49"/>
       <c r="B163" s="1" t="s">
         <v>380</v>
       </c>
@@ -6987,7 +6987,7 @@
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A164" s="34"/>
+      <c r="A164" s="49"/>
       <c r="B164" s="1" t="s">
         <v>381</v>
       </c>
@@ -6996,7 +6996,7 @@
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A165" s="34"/>
+      <c r="A165" s="49"/>
       <c r="B165" s="1" t="s">
         <v>383</v>
       </c>
@@ -7005,7 +7005,7 @@
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A166" s="34"/>
+      <c r="A166" s="49"/>
       <c r="B166" s="1" t="s">
         <v>384</v>
       </c>
@@ -7014,7 +7014,7 @@
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167" s="35"/>
+      <c r="A167" s="50"/>
       <c r="B167" s="1" t="s">
         <v>386</v>
       </c>
@@ -7023,7 +7023,7 @@
       </c>
     </row>
     <row r="168" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="40" t="s">
+      <c r="A168" s="37" t="s">
         <v>388</v>
       </c>
       <c r="B168" s="25" t="s">
@@ -7034,7 +7034,7 @@
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169" s="41"/>
+      <c r="A169" s="38"/>
       <c r="B169" s="9" t="s">
         <v>391</v>
       </c>
@@ -7043,7 +7043,7 @@
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170" s="41"/>
+      <c r="A170" s="38"/>
       <c r="B170" s="9" t="s">
         <v>392</v>
       </c>
@@ -7052,7 +7052,7 @@
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" s="42"/>
+      <c r="A171" s="39"/>
       <c r="B171" s="9" t="s">
         <v>394</v>
       </c>
@@ -7061,7 +7061,7 @@
       </c>
     </row>
     <row r="172" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="43" t="s">
+      <c r="A172" s="33" t="s">
         <v>395</v>
       </c>
       <c r="B172" s="1" t="s">
@@ -7072,7 +7072,7 @@
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173" s="44"/>
+      <c r="A173" s="36"/>
       <c r="B173" s="1" t="s">
         <v>399</v>
       </c>
@@ -7081,7 +7081,7 @@
       </c>
     </row>
     <row r="174" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A174" s="44"/>
+      <c r="A174" s="36"/>
       <c r="B174" s="1" t="s">
         <v>401</v>
       </c>
@@ -7090,7 +7090,7 @@
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A175" s="45"/>
+      <c r="A175" s="34"/>
       <c r="B175" s="1" t="s">
         <v>403</v>
       </c>
@@ -7099,7 +7099,7 @@
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176" s="40" t="s">
+      <c r="A176" s="37" t="s">
         <v>404</v>
       </c>
       <c r="B176" s="9" t="s">
@@ -7110,7 +7110,7 @@
       </c>
     </row>
     <row r="177" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A177" s="41"/>
+      <c r="A177" s="38"/>
       <c r="B177" s="9" t="s">
         <v>407</v>
       </c>
@@ -7119,7 +7119,7 @@
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" s="42"/>
+      <c r="A178" s="39"/>
       <c r="B178" s="9" t="s">
         <v>409</v>
       </c>
@@ -7128,7 +7128,7 @@
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" s="43" t="s">
+      <c r="A179" s="33" t="s">
         <v>410</v>
       </c>
       <c r="B179" s="1" t="s">
@@ -7139,7 +7139,7 @@
       </c>
     </row>
     <row r="180" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A180" s="44"/>
+      <c r="A180" s="36"/>
       <c r="B180" s="8" t="s">
         <v>414</v>
       </c>
@@ -7148,7 +7148,7 @@
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181" s="44"/>
+      <c r="A181" s="36"/>
       <c r="B181" s="1" t="s">
         <v>416</v>
       </c>
@@ -7157,7 +7157,7 @@
       </c>
     </row>
     <row r="182" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A182" s="45"/>
+      <c r="A182" s="34"/>
       <c r="B182" s="1" t="s">
         <v>418</v>
       </c>
@@ -7166,7 +7166,7 @@
       </c>
     </row>
     <row r="183" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="40" t="s">
+      <c r="A183" s="37" t="s">
         <v>419</v>
       </c>
       <c r="B183" s="9" t="s">
@@ -7177,7 +7177,7 @@
       </c>
     </row>
     <row r="184" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A184" s="41"/>
+      <c r="A184" s="38"/>
       <c r="B184" s="9" t="s">
         <v>423</v>
       </c>
@@ -7186,7 +7186,7 @@
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185" s="41"/>
+      <c r="A185" s="38"/>
       <c r="B185" s="9" t="s">
         <v>425</v>
       </c>
@@ -7195,7 +7195,7 @@
       </c>
     </row>
     <row r="186" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A186" s="42"/>
+      <c r="A186" s="39"/>
       <c r="B186" s="9" t="s">
         <v>427</v>
       </c>
@@ -7204,7 +7204,7 @@
       </c>
     </row>
     <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A187" s="43" t="s">
+      <c r="A187" s="33" t="s">
         <v>428</v>
       </c>
       <c r="B187" s="1" t="s">
@@ -7215,7 +7215,7 @@
       </c>
     </row>
     <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A188" s="44"/>
+      <c r="A188" s="36"/>
       <c r="B188" s="1" t="s">
         <v>432</v>
       </c>
@@ -7224,7 +7224,7 @@
       </c>
     </row>
     <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A189" s="45"/>
+      <c r="A189" s="34"/>
       <c r="B189" s="1" t="s">
         <v>434</v>
       </c>
@@ -7233,7 +7233,7 @@
       </c>
     </row>
     <row r="190" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="40" t="s">
+      <c r="A190" s="37" t="s">
         <v>435</v>
       </c>
       <c r="B190" s="9" t="s">
@@ -7244,7 +7244,7 @@
       </c>
     </row>
     <row r="191" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A191" s="41"/>
+      <c r="A191" s="38"/>
       <c r="B191" s="9" t="s">
         <v>439</v>
       </c>
@@ -7253,7 +7253,7 @@
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A192" s="42"/>
+      <c r="A192" s="39"/>
       <c r="B192" s="9" t="s">
         <v>441</v>
       </c>
@@ -7262,7 +7262,7 @@
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A193" s="43" t="s">
+      <c r="A193" s="33" t="s">
         <v>442</v>
       </c>
       <c r="B193" s="1" t="s">
@@ -7273,7 +7273,7 @@
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A194" s="44"/>
+      <c r="A194" s="36"/>
       <c r="B194" s="1" t="s">
         <v>446</v>
       </c>
@@ -7282,7 +7282,7 @@
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A195" s="44"/>
+      <c r="A195" s="36"/>
       <c r="B195" s="1" t="s">
         <v>448</v>
       </c>
@@ -7291,7 +7291,7 @@
       </c>
     </row>
     <row r="196" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A196" s="45"/>
+      <c r="A196" s="34"/>
       <c r="B196" s="1" t="s">
         <v>450</v>
       </c>
@@ -7300,7 +7300,7 @@
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A197" s="40" t="s">
+      <c r="A197" s="37" t="s">
         <v>451</v>
       </c>
       <c r="B197" s="9" t="s">
@@ -7311,7 +7311,7 @@
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A198" s="41"/>
+      <c r="A198" s="38"/>
       <c r="B198" s="9" t="s">
         <v>391</v>
       </c>
@@ -7320,7 +7320,7 @@
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A199" s="41"/>
+      <c r="A199" s="38"/>
       <c r="B199" s="9" t="s">
         <v>392</v>
       </c>
@@ -7329,7 +7329,7 @@
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A200" s="41"/>
+      <c r="A200" s="38"/>
       <c r="B200" s="9" t="s">
         <v>456</v>
       </c>
@@ -7338,7 +7338,7 @@
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A201" s="42"/>
+      <c r="A201" s="39"/>
       <c r="B201" s="9" t="s">
         <v>458</v>
       </c>
@@ -7347,7 +7347,7 @@
       </c>
     </row>
     <row r="202" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="43" t="s">
+      <c r="A202" s="33" t="s">
         <v>459</v>
       </c>
       <c r="B202" s="1" t="s">
@@ -7358,7 +7358,7 @@
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A203" s="44"/>
+      <c r="A203" s="36"/>
       <c r="B203" s="1" t="s">
         <v>463</v>
       </c>
@@ -7367,7 +7367,7 @@
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A204" s="44"/>
+      <c r="A204" s="36"/>
       <c r="B204" s="1" t="s">
         <v>465</v>
       </c>
@@ -7376,7 +7376,7 @@
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A205" s="45"/>
+      <c r="A205" s="34"/>
       <c r="B205" s="1" t="s">
         <v>467</v>
       </c>
@@ -7394,7 +7394,7 @@
       <c r="C206" s="23"/>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A207" s="43" t="s">
+      <c r="A207" s="33" t="s">
         <v>469</v>
       </c>
       <c r="B207" s="1" t="s">
@@ -7405,7 +7405,7 @@
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A208" s="44"/>
+      <c r="A208" s="36"/>
       <c r="B208" s="1" t="s">
         <v>472</v>
       </c>
@@ -7414,7 +7414,7 @@
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A209" s="44"/>
+      <c r="A209" s="36"/>
       <c r="B209" s="1" t="s">
         <v>473</v>
       </c>
@@ -7423,7 +7423,7 @@
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A210" s="44"/>
+      <c r="A210" s="36"/>
       <c r="B210" s="1" t="s">
         <v>475</v>
       </c>
@@ -7432,7 +7432,7 @@
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A211" s="44"/>
+      <c r="A211" s="36"/>
       <c r="B211" s="1" t="s">
         <v>476</v>
       </c>
@@ -7441,7 +7441,7 @@
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A212" s="44"/>
+      <c r="A212" s="36"/>
       <c r="B212" s="1" t="s">
         <v>478</v>
       </c>
@@ -7450,7 +7450,7 @@
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A213" s="44"/>
+      <c r="A213" s="36"/>
       <c r="B213" s="1" t="s">
         <v>480</v>
       </c>
@@ -7459,7 +7459,7 @@
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A214" s="45"/>
+      <c r="A214" s="34"/>
       <c r="B214" s="1" t="s">
         <v>481</v>
       </c>
@@ -7468,7 +7468,7 @@
       </c>
     </row>
     <row r="215" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="40" t="s">
+      <c r="A215" s="37" t="s">
         <v>482</v>
       </c>
       <c r="B215" s="9" t="s">
@@ -7479,7 +7479,7 @@
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A216" s="41"/>
+      <c r="A216" s="38"/>
       <c r="B216" s="9" t="s">
         <v>486</v>
       </c>
@@ -7488,7 +7488,7 @@
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A217" s="41"/>
+      <c r="A217" s="38"/>
       <c r="B217" s="9" t="s">
         <v>487</v>
       </c>
@@ -7497,7 +7497,7 @@
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A218" s="42"/>
+      <c r="A218" s="39"/>
       <c r="B218" s="9" t="s">
         <v>488</v>
       </c>
@@ -7506,7 +7506,7 @@
       </c>
     </row>
     <row r="219" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="43" t="s">
+      <c r="A219" s="33" t="s">
         <v>527</v>
       </c>
       <c r="B219" s="1" t="s">
@@ -7517,7 +7517,7 @@
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A220" s="44"/>
+      <c r="A220" s="36"/>
       <c r="B220" s="1" t="s">
         <v>531</v>
       </c>
@@ -7526,7 +7526,7 @@
       </c>
     </row>
     <row r="221" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A221" s="45"/>
+      <c r="A221" s="34"/>
       <c r="B221" s="1" t="s">
         <v>533</v>
       </c>
@@ -7535,7 +7535,7 @@
       </c>
     </row>
     <row r="222" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="40" t="s">
+      <c r="A222" s="37" t="s">
         <v>534</v>
       </c>
       <c r="B222" s="9" t="s">
@@ -7546,7 +7546,7 @@
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A223" s="41"/>
+      <c r="A223" s="38"/>
       <c r="B223" s="9" t="s">
         <v>538</v>
       </c>
@@ -7555,7 +7555,7 @@
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A224" s="41"/>
+      <c r="A224" s="38"/>
       <c r="B224" s="9" t="s">
         <v>540</v>
       </c>
@@ -7564,7 +7564,7 @@
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A225" s="42"/>
+      <c r="A225" s="39"/>
       <c r="B225" s="9" t="s">
         <v>542</v>
       </c>
@@ -7573,7 +7573,7 @@
       </c>
     </row>
     <row r="226" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="43" t="s">
+      <c r="A226" s="33" t="s">
         <v>543</v>
       </c>
       <c r="B226" s="1" t="s">
@@ -7584,7 +7584,7 @@
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A227" s="44"/>
+      <c r="A227" s="36"/>
       <c r="B227" s="1" t="s">
         <v>546</v>
       </c>
@@ -7593,7 +7593,7 @@
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A228" s="45"/>
+      <c r="A228" s="34"/>
       <c r="B228" s="1" t="s">
         <v>548</v>
       </c>
@@ -7602,7 +7602,7 @@
       </c>
     </row>
     <row r="229" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="40" t="s">
+      <c r="A229" s="37" t="s">
         <v>549</v>
       </c>
       <c r="B229" s="9" t="s">
@@ -7613,7 +7613,7 @@
       </c>
     </row>
     <row r="230" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A230" s="41"/>
+      <c r="A230" s="38"/>
       <c r="B230" s="9" t="s">
         <v>553</v>
       </c>
@@ -7622,7 +7622,7 @@
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A231" s="42"/>
+      <c r="A231" s="39"/>
       <c r="B231" s="9" t="s">
         <v>555</v>
       </c>
@@ -7631,7 +7631,7 @@
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A232" s="43" t="s">
+      <c r="A232" s="33" t="s">
         <v>490</v>
       </c>
       <c r="B232" s="1" t="s">
@@ -7642,7 +7642,7 @@
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A233" s="44"/>
+      <c r="A233" s="36"/>
       <c r="B233" s="1" t="s">
         <v>493</v>
       </c>
@@ -7651,7 +7651,7 @@
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A234" s="44"/>
+      <c r="A234" s="36"/>
       <c r="B234" s="1" t="s">
         <v>495</v>
       </c>
@@ -7660,7 +7660,7 @@
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A235" s="45"/>
+      <c r="A235" s="34"/>
       <c r="B235" s="1" t="s">
         <v>497</v>
       </c>
@@ -7680,7 +7680,7 @@
       </c>
     </row>
     <row r="237" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A237" s="43" t="s">
+      <c r="A237" s="33" t="s">
         <v>501</v>
       </c>
       <c r="B237" s="1" t="s">
@@ -7691,7 +7691,7 @@
       </c>
     </row>
     <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A238" s="44"/>
+      <c r="A238" s="36"/>
       <c r="B238" s="1" t="s">
         <v>505</v>
       </c>
@@ -7700,7 +7700,7 @@
       </c>
     </row>
     <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A239" s="45"/>
+      <c r="A239" s="34"/>
       <c r="B239" s="1" t="s">
         <v>507</v>
       </c>
@@ -7709,7 +7709,7 @@
       </c>
     </row>
     <row r="240" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A240" s="40" t="s">
+      <c r="A240" s="37" t="s">
         <v>508</v>
       </c>
       <c r="B240" s="9" t="s">
@@ -7720,7 +7720,7 @@
       </c>
     </row>
     <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A241" s="42"/>
+      <c r="A241" s="39"/>
       <c r="B241" s="9" t="s">
         <v>512</v>
       </c>
@@ -7729,7 +7729,7 @@
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A242" s="43" t="s">
+      <c r="A242" s="33" t="s">
         <v>513</v>
       </c>
       <c r="B242" s="1" t="s">
@@ -7740,7 +7740,7 @@
       </c>
     </row>
     <row r="243" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A243" s="45"/>
+      <c r="A243" s="34"/>
       <c r="B243" s="1" t="s">
         <v>517</v>
       </c>
@@ -7749,7 +7749,7 @@
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A244" s="40" t="s">
+      <c r="A244" s="37" t="s">
         <v>518</v>
       </c>
       <c r="B244" s="9" t="s">
@@ -7760,7 +7760,7 @@
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A245" s="41"/>
+      <c r="A245" s="38"/>
       <c r="B245" s="9" t="s">
         <v>522</v>
       </c>
@@ -7769,7 +7769,7 @@
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A246" s="41"/>
+      <c r="A246" s="38"/>
       <c r="B246" s="9" t="s">
         <v>524</v>
       </c>
@@ -7778,7 +7778,7 @@
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A247" s="42"/>
+      <c r="A247" s="39"/>
       <c r="B247" s="9" t="s">
         <v>526</v>
       </c>
@@ -7787,7 +7787,7 @@
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A248" s="43" t="s">
+      <c r="A248" s="33" t="s">
         <v>556</v>
       </c>
       <c r="B248" s="1" t="s">
@@ -7798,7 +7798,7 @@
       </c>
     </row>
     <row r="249" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A249" s="44"/>
+      <c r="A249" s="36"/>
       <c r="B249" s="1" t="s">
         <v>560</v>
       </c>
@@ -7807,7 +7807,7 @@
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A250" s="45"/>
+      <c r="A250" s="34"/>
       <c r="B250" s="1" t="s">
         <v>562</v>
       </c>
@@ -7816,7 +7816,7 @@
       </c>
     </row>
     <row r="251" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A251" s="40" t="s">
+      <c r="A251" s="37" t="s">
         <v>563</v>
       </c>
       <c r="B251" s="9" t="s">
@@ -7827,7 +7827,7 @@
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A252" s="41"/>
+      <c r="A252" s="38"/>
       <c r="B252" s="9" t="s">
         <v>566</v>
       </c>
@@ -7836,7 +7836,7 @@
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A253" s="41"/>
+      <c r="A253" s="38"/>
       <c r="B253" s="9" t="s">
         <v>568</v>
       </c>
@@ -7845,7 +7845,7 @@
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A254" s="42"/>
+      <c r="A254" s="39"/>
       <c r="B254" s="9" t="s">
         <v>570</v>
       </c>
@@ -7865,7 +7865,7 @@
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A256" s="43" t="s">
+      <c r="A256" s="33" t="s">
         <v>575</v>
       </c>
       <c r="B256" s="1" t="s">
@@ -7876,7 +7876,7 @@
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A257" s="44"/>
+      <c r="A257" s="36"/>
       <c r="B257" s="1" t="s">
         <v>579</v>
       </c>
@@ -7885,7 +7885,7 @@
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A258" s="44"/>
+      <c r="A258" s="36"/>
       <c r="B258" s="1" t="s">
         <v>581</v>
       </c>
@@ -7894,7 +7894,7 @@
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A259" s="45"/>
+      <c r="A259" s="34"/>
       <c r="B259" s="1" t="s">
         <v>583</v>
       </c>
@@ -7903,7 +7903,7 @@
       </c>
     </row>
     <row r="260" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A260" s="43" t="s">
+      <c r="A260" s="33" t="s">
         <v>584</v>
       </c>
       <c r="B260" s="1" t="s">
@@ -7914,7 +7914,7 @@
       </c>
     </row>
     <row r="261" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A261" s="45"/>
+      <c r="A261" s="34"/>
       <c r="B261" s="1" t="s">
         <v>588</v>
       </c>
@@ -8057,7 +8057,7 @@
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A276" s="39" t="s">
+      <c r="A276" s="40" t="s">
         <v>166</v>
       </c>
       <c r="B276" s="1" t="s">
@@ -8068,14 +8068,14 @@
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A277" s="39"/>
+      <c r="A277" s="40"/>
       <c r="B277" s="1" t="s">
         <v>163</v>
       </c>
       <c r="C277" s="1"/>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A278" s="39"/>
+      <c r="A278" s="40"/>
       <c r="B278" s="1" t="s">
         <v>164</v>
       </c>
@@ -8100,7 +8100,7 @@
       <c r="C280" s="1"/>
     </row>
     <row r="281" spans="1:3" ht="180" x14ac:dyDescent="0.25">
-      <c r="A281" s="43" t="s">
+      <c r="A281" s="33" t="s">
         <v>600</v>
       </c>
       <c r="B281" s="1" t="s">
@@ -8111,23 +8111,23 @@
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A282" s="44"/>
+      <c r="A282" s="36"/>
       <c r="B282" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C282" s="38" t="s">
+      <c r="C282" s="35" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A283" s="44"/>
+      <c r="A283" s="36"/>
       <c r="B283" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C283" s="38"/>
+      <c r="C283" s="35"/>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A284" s="44"/>
+      <c r="A284" s="36"/>
       <c r="B284" s="1" t="s">
         <v>183</v>
       </c>
@@ -8136,7 +8136,7 @@
       </c>
     </row>
     <row r="285" spans="1:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="A285" s="45"/>
+      <c r="A285" s="34"/>
       <c r="B285" s="1" t="s">
         <v>598</v>
       </c>
@@ -8156,7 +8156,7 @@
       </c>
     </row>
     <row r="287" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A287" s="33" t="s">
+      <c r="A287" s="48" t="s">
         <v>602</v>
       </c>
       <c r="B287" s="21" t="s">
@@ -8167,7 +8167,7 @@
       </c>
     </row>
     <row r="288" spans="1:3" ht="135" x14ac:dyDescent="0.25">
-      <c r="A288" s="34"/>
+      <c r="A288" s="49"/>
       <c r="B288" s="21" t="s">
         <v>605</v>
       </c>
@@ -8176,7 +8176,7 @@
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A289" s="34"/>
+      <c r="A289" s="49"/>
       <c r="B289" s="21" t="s">
         <v>608</v>
       </c>
@@ -8185,7 +8185,7 @@
       </c>
     </row>
     <row r="290" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A290" s="34"/>
+      <c r="A290" s="49"/>
       <c r="B290" s="21" t="s">
         <v>609</v>
       </c>
@@ -8194,7 +8194,7 @@
       </c>
     </row>
     <row r="291" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A291" s="34"/>
+      <c r="A291" s="49"/>
       <c r="B291" s="21" t="s">
         <v>610</v>
       </c>
@@ -8203,7 +8203,7 @@
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A292" s="35"/>
+      <c r="A292" s="50"/>
       <c r="B292" s="21" t="s">
         <v>614</v>
       </c>
@@ -8214,6 +8214,62 @@
   </sheetData>
   <autoFilter ref="A1:C286" xr:uid="{7416C5AA-AA6E-41AB-BBA6-B527D527C8A0}"/>
   <mergeCells count="72">
+    <mergeCell ref="A287:A292"/>
+    <mergeCell ref="A8:A16"/>
+    <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A32:A50"/>
+    <mergeCell ref="A159:A167"/>
+    <mergeCell ref="A168:A171"/>
+    <mergeCell ref="A172:A175"/>
+    <mergeCell ref="A276:A278"/>
+    <mergeCell ref="A248:A250"/>
+    <mergeCell ref="A232:A235"/>
+    <mergeCell ref="A237:A239"/>
+    <mergeCell ref="A240:A241"/>
+    <mergeCell ref="A242:A243"/>
+    <mergeCell ref="A244:A247"/>
+    <mergeCell ref="A193:A196"/>
+    <mergeCell ref="A197:A201"/>
+    <mergeCell ref="A202:A205"/>
+    <mergeCell ref="A207:A214"/>
+    <mergeCell ref="A272:A273"/>
+    <mergeCell ref="A256:A259"/>
+    <mergeCell ref="A260:A261"/>
+    <mergeCell ref="A147:A151"/>
+    <mergeCell ref="A215:A218"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A182"/>
+    <mergeCell ref="A183:A186"/>
+    <mergeCell ref="A187:A189"/>
+    <mergeCell ref="A190:A192"/>
+    <mergeCell ref="A251:A254"/>
+    <mergeCell ref="A219:A221"/>
+    <mergeCell ref="A222:A225"/>
+    <mergeCell ref="A226:A228"/>
+    <mergeCell ref="A229:A231"/>
+    <mergeCell ref="A152:A158"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="A102:A106"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="A100:A101"/>
+    <mergeCell ref="A126:A128"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A114"/>
+    <mergeCell ref="A72:A76"/>
+    <mergeCell ref="A77:A80"/>
+    <mergeCell ref="A97:A99"/>
+    <mergeCell ref="A120:A123"/>
+    <mergeCell ref="A124:A125"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="C282:C283"/>
     <mergeCell ref="A281:A285"/>
@@ -8230,62 +8286,6 @@
     <mergeCell ref="A61:A67"/>
     <mergeCell ref="A68:A69"/>
     <mergeCell ref="A70:A71"/>
-    <mergeCell ref="A72:A76"/>
-    <mergeCell ref="A77:A80"/>
-    <mergeCell ref="A97:A99"/>
-    <mergeCell ref="A120:A123"/>
-    <mergeCell ref="A124:A125"/>
-    <mergeCell ref="A126:A128"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="A129:A130"/>
-    <mergeCell ref="A115:A116"/>
-    <mergeCell ref="A117:A119"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A114"/>
-    <mergeCell ref="C84:C85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="A91:A92"/>
-    <mergeCell ref="A93:A94"/>
-    <mergeCell ref="A102:A106"/>
-    <mergeCell ref="A95:A96"/>
-    <mergeCell ref="A100:A101"/>
-    <mergeCell ref="A272:A273"/>
-    <mergeCell ref="A256:A259"/>
-    <mergeCell ref="A260:A261"/>
-    <mergeCell ref="A147:A151"/>
-    <mergeCell ref="A215:A218"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A182"/>
-    <mergeCell ref="A183:A186"/>
-    <mergeCell ref="A187:A189"/>
-    <mergeCell ref="A190:A192"/>
-    <mergeCell ref="A251:A254"/>
-    <mergeCell ref="A219:A221"/>
-    <mergeCell ref="A222:A225"/>
-    <mergeCell ref="A226:A228"/>
-    <mergeCell ref="A229:A231"/>
-    <mergeCell ref="A152:A158"/>
-    <mergeCell ref="A244:A247"/>
-    <mergeCell ref="A193:A196"/>
-    <mergeCell ref="A197:A201"/>
-    <mergeCell ref="A202:A205"/>
-    <mergeCell ref="A207:A214"/>
-    <mergeCell ref="A287:A292"/>
-    <mergeCell ref="A8:A16"/>
-    <mergeCell ref="A23:A27"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="A32:A50"/>
-    <mergeCell ref="A159:A167"/>
-    <mergeCell ref="A168:A171"/>
-    <mergeCell ref="A172:A175"/>
-    <mergeCell ref="A276:A278"/>
-    <mergeCell ref="A248:A250"/>
-    <mergeCell ref="A232:A235"/>
-    <mergeCell ref="A237:A239"/>
-    <mergeCell ref="A240:A241"/>
-    <mergeCell ref="A242:A243"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
ajout de la partie AWS
</commit_message>
<xml_diff>
--- a/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
+++ b/KUBERNETES/Kubernetes_liste_des_commandes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a5f61b3e4cd8107/Inès_perso/M2i_administraeur_CLOUD.0.0/Cours_Python_M2i/KUBERNETES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2410" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{334E8C58-A663-4A65-B402-4BE34D0BDBD7}"/>
+  <xr:revisionPtr revIDLastSave="2412" documentId="8_{4309FA21-DA46-4726-B3AF-5F415FC36ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D317B7D-6E86-4244-8152-AE2A9DCDA1BF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8D2D9E53-07E4-4E8B-82A4-55704ED06D6A}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="625">
   <si>
     <t>Commandes</t>
   </si>
@@ -4704,9 +4704,6 @@
     <t>Demander au conteneur son nom d'hôte :</t>
   </si>
   <si>
-    <t xml:space="preserve">Céer un service </t>
-  </si>
-  <si>
     <t>kubectl expose deployment storefront -n practice-observe --port=80</t>
   </si>
   <si>
@@ -4789,6 +4786,12 @@
   </si>
   <si>
     <t>Cette commande crée un Service nommé storefront à partir du Deployment</t>
+  </si>
+  <si>
+    <t>²</t>
+  </si>
+  <si>
+    <t>kubectl create namespace &lt;nom_donné&gt;</t>
   </si>
 </sst>
 </file>
@@ -5028,16 +5031,22 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5060,12 +5069,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5460,7 +5463,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="36" t="s">
         <v>174</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -5471,7 +5474,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
+      <c r="A4" s="38"/>
       <c r="B4" s="7" t="s">
         <v>358</v>
       </c>
@@ -5491,27 +5494,27 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="33" t="s">
+        <v>623</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="34"/>
+      <c r="B7" s="1" t="s">
         <v>620</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A7" s="45"/>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>621</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>622</v>
-      </c>
     </row>
     <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="43" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="9" t="s">
@@ -5522,7 +5525,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="41"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="9" t="s">
         <v>172</v>
       </c>
@@ -5531,7 +5534,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="41"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="9" t="s">
         <v>54</v>
       </c>
@@ -5540,7 +5543,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="41"/>
+      <c r="A11" s="43"/>
       <c r="B11" s="9" t="s">
         <v>56</v>
       </c>
@@ -5549,7 +5552,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="41"/>
+      <c r="A12" s="43"/>
       <c r="B12" s="9" t="s">
         <v>58</v>
       </c>
@@ -5558,7 +5561,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="41"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="9" t="s">
         <v>59</v>
       </c>
@@ -5567,7 +5570,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="41"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="9" t="s">
         <v>62</v>
       </c>
@@ -5576,7 +5579,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="41"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="9" t="s">
         <v>10</v>
       </c>
@@ -5585,7 +5588,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="41"/>
+      <c r="A16" s="43"/>
       <c r="B16" s="9" t="s">
         <v>4</v>
       </c>
@@ -5594,7 +5597,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="42" t="s">
         <v>187</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -5605,7 +5608,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="42"/>
       <c r="B18" s="1" t="s">
         <v>6</v>
       </c>
@@ -5614,7 +5617,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="42"/>
       <c r="B19" s="1" t="s">
         <v>73</v>
       </c>
@@ -5623,14 +5626,14 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="42"/>
       <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
       <c r="C20" s="35"/>
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="40"/>
+      <c r="A21" s="42"/>
       <c r="B21" s="1" t="s">
         <v>17</v>
       </c>
@@ -5639,7 +5642,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="40"/>
+      <c r="A22" s="42"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -5659,7 +5662,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="41"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="9" t="s">
         <v>8</v>
       </c>
@@ -5668,7 +5671,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="41"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="9" t="s">
         <v>68</v>
       </c>
@@ -5677,7 +5680,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="41"/>
+      <c r="A26" s="43"/>
       <c r="B26" s="9" t="s">
         <v>22</v>
       </c>
@@ -5686,7 +5689,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="41"/>
+      <c r="A27" s="43"/>
       <c r="B27" s="9" t="s">
         <v>69</v>
       </c>
@@ -5695,7 +5698,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="42" t="s">
         <v>188</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -5706,7 +5709,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="42"/>
       <c r="B29" s="1" t="s">
         <v>212</v>
       </c>
@@ -5715,7 +5718,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="1" t="s">
         <v>84</v>
       </c>
@@ -5724,7 +5727,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="40"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="1" t="s">
         <v>144</v>
       </c>
@@ -5733,7 +5736,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="37" t="s">
+      <c r="A32" s="39" t="s">
         <v>197</v>
       </c>
       <c r="B32" s="9" t="s">
@@ -5744,7 +5747,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="38"/>
+      <c r="A33" s="40"/>
       <c r="B33" s="9" t="s">
         <v>190</v>
       </c>
@@ -5753,7 +5756,7 @@
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="38"/>
+      <c r="A34" s="40"/>
       <c r="B34" s="9" t="s">
         <v>86</v>
       </c>
@@ -5762,7 +5765,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="38"/>
+      <c r="A35" s="40"/>
       <c r="B35" s="9" t="s">
         <v>64</v>
       </c>
@@ -5771,7 +5774,7 @@
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="38"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="9" t="s">
         <v>88</v>
       </c>
@@ -5780,7 +5783,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A37" s="38"/>
+      <c r="A37" s="40"/>
       <c r="B37" s="9" t="s">
         <v>20</v>
       </c>
@@ -5789,7 +5792,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="38"/>
+      <c r="A38" s="40"/>
       <c r="B38" s="9" t="s">
         <v>90</v>
       </c>
@@ -5798,14 +5801,14 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="38"/>
+      <c r="A39" s="40"/>
       <c r="B39" s="9" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="9"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="38"/>
+      <c r="A40" s="40"/>
       <c r="B40" s="9" t="s">
         <v>91</v>
       </c>
@@ -5814,7 +5817,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="38"/>
+      <c r="A41" s="40"/>
       <c r="B41" s="9" t="s">
         <v>94</v>
       </c>
@@ -5823,7 +5826,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="38"/>
+      <c r="A42" s="40"/>
       <c r="B42" s="9" t="s">
         <v>92</v>
       </c>
@@ -5832,7 +5835,7 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="38"/>
+      <c r="A43" s="40"/>
       <c r="B43" s="9" t="s">
         <v>14</v>
       </c>
@@ -5841,7 +5844,7 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="38"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="9" t="s">
         <v>15</v>
       </c>
@@ -5850,7 +5853,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A45" s="38"/>
+      <c r="A45" s="40"/>
       <c r="B45" s="9" t="s">
         <v>19</v>
       </c>
@@ -5859,7 +5862,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A46" s="38"/>
+      <c r="A46" s="40"/>
       <c r="B46" s="9" t="s">
         <v>571</v>
       </c>
@@ -5868,7 +5871,7 @@
       </c>
     </row>
     <row r="47" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A47" s="38"/>
+      <c r="A47" s="40"/>
       <c r="B47" s="9" t="s">
         <v>589</v>
       </c>
@@ -5877,7 +5880,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="38"/>
+      <c r="A48" s="40"/>
       <c r="B48" s="9" t="s">
         <v>591</v>
       </c>
@@ -5886,7 +5889,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="38"/>
+      <c r="A49" s="40"/>
       <c r="B49" s="9" t="s">
         <v>592</v>
       </c>
@@ -5895,7 +5898,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="39"/>
+      <c r="A50" s="41"/>
       <c r="B50" s="9" t="s">
         <v>93</v>
       </c>
@@ -5904,7 +5907,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="42" t="s">
         <v>198</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -5915,7 +5918,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="40"/>
+      <c r="A52" s="42"/>
       <c r="B52" s="1" t="s">
         <v>96</v>
       </c>
@@ -5924,7 +5927,7 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="40"/>
+      <c r="A53" s="42"/>
       <c r="B53" s="1" t="s">
         <v>98</v>
       </c>
@@ -5933,7 +5936,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="40"/>
+      <c r="A54" s="42"/>
       <c r="B54" s="1" t="s">
         <v>71</v>
       </c>
@@ -5942,7 +5945,7 @@
       </c>
     </row>
     <row r="55" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="40"/>
+      <c r="A55" s="42"/>
       <c r="B55" s="1" t="s">
         <v>18</v>
       </c>
@@ -5951,7 +5954,7 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A56" s="40"/>
+      <c r="A56" s="42"/>
       <c r="B56" s="1" t="s">
         <v>99</v>
       </c>
@@ -5960,7 +5963,7 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="41" t="s">
+      <c r="A57" s="43" t="s">
         <v>199</v>
       </c>
       <c r="B57" s="9" t="s">
@@ -5971,7 +5974,7 @@
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="41"/>
+      <c r="A58" s="43"/>
       <c r="B58" s="9" t="s">
         <v>101</v>
       </c>
@@ -5980,7 +5983,7 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="41"/>
+      <c r="A59" s="43"/>
       <c r="B59" s="9" t="s">
         <v>103</v>
       </c>
@@ -5989,7 +5992,7 @@
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="41"/>
+      <c r="A60" s="43"/>
       <c r="B60" s="9" t="s">
         <v>106</v>
       </c>
@@ -5998,7 +6001,7 @@
       </c>
     </row>
     <row r="61" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A61" s="40" t="s">
+      <c r="A61" s="42" t="s">
         <v>200</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -6009,7 +6012,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="40"/>
+      <c r="A62" s="42"/>
       <c r="B62" s="1" t="s">
         <v>107</v>
       </c>
@@ -6018,7 +6021,7 @@
       </c>
     </row>
     <row r="63" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A63" s="40"/>
+      <c r="A63" s="42"/>
       <c r="B63" s="1" t="s">
         <v>110</v>
       </c>
@@ -6027,7 +6030,7 @@
       </c>
     </row>
     <row r="64" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64" s="40"/>
+      <c r="A64" s="42"/>
       <c r="B64" s="1" t="s">
         <v>26</v>
       </c>
@@ -6036,7 +6039,7 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="40"/>
+      <c r="A65" s="42"/>
       <c r="B65" s="1" t="s">
         <v>36</v>
       </c>
@@ -6045,7 +6048,7 @@
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="40"/>
+      <c r="A66" s="42"/>
       <c r="B66" s="1" t="s">
         <v>148</v>
       </c>
@@ -6054,7 +6057,7 @@
       </c>
     </row>
     <row r="67" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A67" s="40"/>
+      <c r="A67" s="42"/>
       <c r="B67" s="1" t="s">
         <v>50</v>
       </c>
@@ -6063,7 +6066,7 @@
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="43" t="s">
         <v>203</v>
       </c>
       <c r="B68" s="9" t="s">
@@ -6074,7 +6077,7 @@
       </c>
     </row>
     <row r="69" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="41"/>
+      <c r="A69" s="43"/>
       <c r="B69" s="9" t="s">
         <v>114</v>
       </c>
@@ -6083,7 +6086,7 @@
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="40" t="s">
+      <c r="A70" s="42" t="s">
         <v>204</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -6094,7 +6097,7 @@
       </c>
     </row>
     <row r="71" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="40"/>
+      <c r="A71" s="42"/>
       <c r="B71" s="1" t="s">
         <v>122</v>
       </c>
@@ -6103,7 +6106,7 @@
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="41" t="s">
+      <c r="A72" s="43" t="s">
         <v>205</v>
       </c>
       <c r="B72" s="9" t="s">
@@ -6114,7 +6117,7 @@
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="41"/>
+      <c r="A73" s="43"/>
       <c r="B73" s="9" t="s">
         <v>126</v>
       </c>
@@ -6123,7 +6126,7 @@
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="41"/>
+      <c r="A74" s="43"/>
       <c r="B74" s="9" t="s">
         <v>128</v>
       </c>
@@ -6132,7 +6135,7 @@
       </c>
     </row>
     <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A75" s="41"/>
+      <c r="A75" s="43"/>
       <c r="B75" s="9" t="s">
         <v>615</v>
       </c>
@@ -6141,7 +6144,7 @@
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="41"/>
+      <c r="A76" s="43"/>
       <c r="B76" s="9" t="s">
         <v>130</v>
       </c>
@@ -6150,7 +6153,7 @@
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" s="40" t="s">
+      <c r="A77" s="42" t="s">
         <v>206</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -6161,7 +6164,7 @@
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="40"/>
+      <c r="A78" s="42"/>
       <c r="B78" s="1" t="s">
         <v>134</v>
       </c>
@@ -6170,7 +6173,7 @@
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="40"/>
+      <c r="A79" s="42"/>
       <c r="B79" s="1" t="s">
         <v>617</v>
       </c>
@@ -6179,7 +6182,7 @@
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" s="40"/>
+      <c r="A80" s="42"/>
       <c r="B80" s="1" t="s">
         <v>136</v>
       </c>
@@ -6188,7 +6191,7 @@
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" s="41" t="s">
+      <c r="A81" s="43" t="s">
         <v>207</v>
       </c>
       <c r="B81" s="9" t="s">
@@ -6199,7 +6202,7 @@
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="41"/>
+      <c r="A82" s="43"/>
       <c r="B82" s="9" t="s">
         <v>139</v>
       </c>
@@ -6217,25 +6220,25 @@
       <c r="C83" s="1"/>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" s="37" t="s">
+      <c r="A84" s="39" t="s">
         <v>215</v>
       </c>
       <c r="B84" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="C84" s="42" t="s">
+      <c r="C84" s="44" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="39"/>
+      <c r="A85" s="41"/>
       <c r="B85" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C85" s="43"/>
+      <c r="C85" s="45"/>
     </row>
     <row r="86" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="33" t="s">
+      <c r="A86" s="36" t="s">
         <v>219</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -6246,7 +6249,7 @@
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="36"/>
+      <c r="A87" s="37"/>
       <c r="B87" s="1" t="s">
         <v>156</v>
       </c>
@@ -6255,7 +6258,7 @@
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" s="36"/>
+      <c r="A88" s="37"/>
       <c r="B88" s="1" t="s">
         <v>157</v>
       </c>
@@ -6264,7 +6267,7 @@
       </c>
     </row>
     <row r="89" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A89" s="34"/>
+      <c r="A89" s="38"/>
       <c r="B89" s="1" t="s">
         <v>220</v>
       </c>
@@ -6284,7 +6287,7 @@
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="33" t="s">
+      <c r="A91" s="36" t="s">
         <v>228</v>
       </c>
       <c r="B91" s="1" t="s">
@@ -6295,7 +6298,7 @@
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" s="34"/>
+      <c r="A92" s="38"/>
       <c r="B92" s="1" t="s">
         <v>227</v>
       </c>
@@ -6304,7 +6307,7 @@
       </c>
     </row>
     <row r="93" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="37" t="s">
+      <c r="A93" s="39" t="s">
         <v>233</v>
       </c>
       <c r="B93" s="9" t="s">
@@ -6315,7 +6318,7 @@
       </c>
     </row>
     <row r="94" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A94" s="39"/>
+      <c r="A94" s="41"/>
       <c r="B94" s="9" t="s">
         <v>232</v>
       </c>
@@ -6324,7 +6327,7 @@
       </c>
     </row>
     <row r="95" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="33" t="s">
+      <c r="A95" s="36" t="s">
         <v>234</v>
       </c>
       <c r="B95" s="1" t="s">
@@ -6335,7 +6338,7 @@
       </c>
     </row>
     <row r="96" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A96" s="34"/>
+      <c r="A96" s="38"/>
       <c r="B96" s="1" t="s">
         <v>237</v>
       </c>
@@ -6344,7 +6347,7 @@
       </c>
     </row>
     <row r="97" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="37" t="s">
+      <c r="A97" s="39" t="s">
         <v>239</v>
       </c>
       <c r="B97" s="9" t="s">
@@ -6355,7 +6358,7 @@
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98" s="38"/>
+      <c r="A98" s="40"/>
       <c r="B98" s="9" t="s">
         <v>243</v>
       </c>
@@ -6364,7 +6367,7 @@
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A99" s="39"/>
+      <c r="A99" s="41"/>
       <c r="B99" s="9" t="s">
         <v>245</v>
       </c>
@@ -6373,7 +6376,7 @@
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A100" s="44" t="s">
+      <c r="A100" s="33" t="s">
         <v>246</v>
       </c>
       <c r="B100" s="1" t="s">
@@ -6384,7 +6387,7 @@
       </c>
     </row>
     <row r="101" spans="1:3" ht="270" x14ac:dyDescent="0.25">
-      <c r="A101" s="45"/>
+      <c r="A101" s="34"/>
       <c r="B101" s="1" t="s">
         <v>250</v>
       </c>
@@ -6393,7 +6396,7 @@
       </c>
     </row>
     <row r="102" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="37" t="s">
+      <c r="A102" s="39" t="s">
         <v>261</v>
       </c>
       <c r="B102" s="9" t="s">
@@ -6404,7 +6407,7 @@
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" s="38"/>
+      <c r="A103" s="40"/>
       <c r="B103" s="9" t="s">
         <v>254</v>
       </c>
@@ -6413,7 +6416,7 @@
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" s="38"/>
+      <c r="A104" s="40"/>
       <c r="B104" s="9" t="s">
         <v>256</v>
       </c>
@@ -6422,7 +6425,7 @@
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A105" s="38"/>
+      <c r="A105" s="40"/>
       <c r="B105" s="9" t="s">
         <v>257</v>
       </c>
@@ -6431,7 +6434,7 @@
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106" s="39"/>
+      <c r="A106" s="41"/>
       <c r="B106" s="9" t="s">
         <v>260</v>
       </c>
@@ -6440,7 +6443,7 @@
       </c>
     </row>
     <row r="107" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="33" t="s">
+      <c r="A107" s="36" t="s">
         <v>262</v>
       </c>
       <c r="B107" s="1" t="s">
@@ -6451,7 +6454,7 @@
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A108" s="36"/>
+      <c r="A108" s="37"/>
       <c r="B108" s="1" t="s">
         <v>266</v>
       </c>
@@ -6460,7 +6463,7 @@
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109" s="34"/>
+      <c r="A109" s="38"/>
       <c r="B109" s="1" t="s">
         <v>267</v>
       </c>
@@ -6469,7 +6472,7 @@
       </c>
     </row>
     <row r="110" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="37" t="s">
+      <c r="A110" s="39" t="s">
         <v>279</v>
       </c>
       <c r="B110" s="9" t="s">
@@ -6480,7 +6483,7 @@
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A111" s="38"/>
+      <c r="A111" s="40"/>
       <c r="B111" s="9" t="s">
         <v>272</v>
       </c>
@@ -6489,7 +6492,7 @@
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A112" s="38"/>
+      <c r="A112" s="40"/>
       <c r="B112" s="9" t="s">
         <v>273</v>
       </c>
@@ -6498,7 +6501,7 @@
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A113" s="38"/>
+      <c r="A113" s="40"/>
       <c r="B113" s="9" t="s">
         <v>275</v>
       </c>
@@ -6507,7 +6510,7 @@
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="39"/>
+      <c r="A114" s="41"/>
       <c r="B114" s="9" t="s">
         <v>278</v>
       </c>
@@ -6516,7 +6519,7 @@
       </c>
     </row>
     <row r="115" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="33" t="s">
+      <c r="A115" s="36" t="s">
         <v>280</v>
       </c>
       <c r="B115" s="1" t="s">
@@ -6527,7 +6530,7 @@
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116" s="34"/>
+      <c r="A116" s="38"/>
       <c r="B116" s="1" t="s">
         <v>284</v>
       </c>
@@ -6536,7 +6539,7 @@
       </c>
     </row>
     <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A117" s="37" t="s">
+      <c r="A117" s="39" t="s">
         <v>285</v>
       </c>
       <c r="B117" s="9" t="s">
@@ -6547,7 +6550,7 @@
       </c>
     </row>
     <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A118" s="38"/>
+      <c r="A118" s="40"/>
       <c r="B118" s="9" t="s">
         <v>289</v>
       </c>
@@ -6556,7 +6559,7 @@
       </c>
     </row>
     <row r="119" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A119" s="39"/>
+      <c r="A119" s="41"/>
       <c r="B119" s="9" t="s">
         <v>291</v>
       </c>
@@ -6565,7 +6568,7 @@
       </c>
     </row>
     <row r="120" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="33" t="s">
+      <c r="A120" s="36" t="s">
         <v>292</v>
       </c>
       <c r="B120" s="1" t="s">
@@ -6576,7 +6579,7 @@
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121" s="36"/>
+      <c r="A121" s="37"/>
       <c r="B121" s="1" t="s">
         <v>296</v>
       </c>
@@ -6585,7 +6588,7 @@
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A122" s="36"/>
+      <c r="A122" s="37"/>
       <c r="B122" s="1" t="s">
         <v>298</v>
       </c>
@@ -6594,7 +6597,7 @@
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A123" s="34"/>
+      <c r="A123" s="38"/>
       <c r="B123" s="1" t="s">
         <v>300</v>
       </c>
@@ -6603,7 +6606,7 @@
       </c>
     </row>
     <row r="124" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="37" t="s">
+      <c r="A124" s="39" t="s">
         <v>301</v>
       </c>
       <c r="B124" s="9" t="s">
@@ -6614,7 +6617,7 @@
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A125" s="39"/>
+      <c r="A125" s="41"/>
       <c r="B125" s="9" t="s">
         <v>305</v>
       </c>
@@ -6623,7 +6626,7 @@
       </c>
     </row>
     <row r="126" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="33" t="s">
+      <c r="A126" s="36" t="s">
         <v>306</v>
       </c>
       <c r="B126" s="1" t="s">
@@ -6634,7 +6637,7 @@
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127" s="36"/>
+      <c r="A127" s="37"/>
       <c r="B127" s="1" t="s">
         <v>309</v>
       </c>
@@ -6643,7 +6646,7 @@
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128" s="34"/>
+      <c r="A128" s="38"/>
       <c r="B128" s="1" t="s">
         <v>311</v>
       </c>
@@ -6652,7 +6655,7 @@
       </c>
     </row>
     <row r="129" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="37" t="s">
+      <c r="A129" s="39" t="s">
         <v>312</v>
       </c>
       <c r="B129" s="9" t="s">
@@ -6663,7 +6666,7 @@
       </c>
     </row>
     <row r="130" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A130" s="39"/>
+      <c r="A130" s="41"/>
       <c r="B130" s="9" t="s">
         <v>315</v>
       </c>
@@ -6681,7 +6684,7 @@
       </c>
     </row>
     <row r="132" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="37" t="s">
+      <c r="A132" s="39" t="s">
         <v>319</v>
       </c>
       <c r="B132" s="9" t="s">
@@ -6692,7 +6695,7 @@
       </c>
     </row>
     <row r="133" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A133" s="38"/>
+      <c r="A133" s="40"/>
       <c r="B133" s="8" t="s">
         <v>323</v>
       </c>
@@ -6701,7 +6704,7 @@
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" s="39"/>
+      <c r="A134" s="41"/>
       <c r="B134" s="9" t="s">
         <v>325</v>
       </c>
@@ -6710,7 +6713,7 @@
       </c>
     </row>
     <row r="135" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="33" t="s">
+      <c r="A135" s="36" t="s">
         <v>326</v>
       </c>
       <c r="B135" s="1" t="s">
@@ -6721,7 +6724,7 @@
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A136" s="34"/>
+      <c r="A136" s="38"/>
       <c r="B136" s="1" t="s">
         <v>330</v>
       </c>
@@ -6730,7 +6733,7 @@
       </c>
     </row>
     <row r="137" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="37" t="s">
+      <c r="A137" s="39" t="s">
         <v>338</v>
       </c>
       <c r="B137" s="9" t="s">
@@ -6741,7 +6744,7 @@
       </c>
     </row>
     <row r="138" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A138" s="39"/>
+      <c r="A138" s="41"/>
       <c r="B138" s="9" t="s">
         <v>334</v>
       </c>
@@ -6750,7 +6753,7 @@
       </c>
     </row>
     <row r="139" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="33" t="s">
+      <c r="A139" s="36" t="s">
         <v>339</v>
       </c>
       <c r="B139" s="1" t="s">
@@ -6761,7 +6764,7 @@
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A140" s="34"/>
+      <c r="A140" s="38"/>
       <c r="B140" s="1" t="s">
         <v>328</v>
       </c>
@@ -6770,7 +6773,7 @@
       </c>
     </row>
     <row r="141" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A141" s="37" t="s">
+      <c r="A141" s="39" t="s">
         <v>344</v>
       </c>
       <c r="B141" s="9" t="s">
@@ -6781,7 +6784,7 @@
       </c>
     </row>
     <row r="142" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="39"/>
+      <c r="A142" s="41"/>
       <c r="B142" s="25" t="s">
         <v>343</v>
       </c>
@@ -6801,7 +6804,7 @@
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A144" s="37" t="s">
+      <c r="A144" s="39" t="s">
         <v>353</v>
       </c>
       <c r="B144" s="25" t="s">
@@ -6812,7 +6815,7 @@
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" s="38"/>
+      <c r="A145" s="40"/>
       <c r="B145" s="9" t="s">
         <v>350</v>
       </c>
@@ -6821,7 +6824,7 @@
       </c>
     </row>
     <row r="146" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="39"/>
+      <c r="A146" s="41"/>
       <c r="B146" s="25" t="s">
         <v>352</v>
       </c>
@@ -6830,18 +6833,18 @@
       </c>
     </row>
     <row r="147" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="33" t="s">
+      <c r="A147" s="36" t="s">
         <v>354</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>154</v>
+        <v>624</v>
       </c>
       <c r="C147" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="36"/>
+      <c r="A148" s="37"/>
       <c r="B148" s="1" t="s">
         <v>156</v>
       </c>
@@ -6850,7 +6853,7 @@
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" s="36"/>
+      <c r="A149" s="37"/>
       <c r="B149" s="1" t="s">
         <v>157</v>
       </c>
@@ -6859,7 +6862,7 @@
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150" s="36"/>
+      <c r="A150" s="37"/>
       <c r="B150" s="1" t="s">
         <v>159</v>
       </c>
@@ -6868,14 +6871,14 @@
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151" s="34"/>
+      <c r="A151" s="38"/>
       <c r="B151" s="1" t="s">
         <v>160</v>
       </c>
       <c r="C151" s="19"/>
     </row>
     <row r="152" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="37" t="s">
+      <c r="A152" s="39" t="s">
         <v>359</v>
       </c>
       <c r="B152" s="9" t="s">
@@ -6886,7 +6889,7 @@
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153" s="38"/>
+      <c r="A153" s="40"/>
       <c r="B153" s="9" t="s">
         <v>362</v>
       </c>
@@ -6895,7 +6898,7 @@
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154" s="38"/>
+      <c r="A154" s="40"/>
       <c r="B154" s="29" t="s">
         <v>365</v>
       </c>
@@ -6904,7 +6907,7 @@
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155" s="38"/>
+      <c r="A155" s="40"/>
       <c r="B155" s="9" t="s">
         <v>367</v>
       </c>
@@ -6913,7 +6916,7 @@
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A156" s="38"/>
+      <c r="A156" s="40"/>
       <c r="B156" s="9" t="s">
         <v>369</v>
       </c>
@@ -6922,7 +6925,7 @@
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157" s="38"/>
+      <c r="A157" s="40"/>
       <c r="B157" s="9" t="s">
         <v>371</v>
       </c>
@@ -6931,7 +6934,7 @@
       </c>
     </row>
     <row r="158" spans="1:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="A158" s="39"/>
+      <c r="A158" s="41"/>
       <c r="B158" s="9" t="s">
         <v>373</v>
       </c>
@@ -7023,7 +7026,7 @@
       </c>
     </row>
     <row r="168" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="37" t="s">
+      <c r="A168" s="39" t="s">
         <v>388</v>
       </c>
       <c r="B168" s="25" t="s">
@@ -7034,7 +7037,7 @@
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169" s="38"/>
+      <c r="A169" s="40"/>
       <c r="B169" s="9" t="s">
         <v>391</v>
       </c>
@@ -7043,7 +7046,7 @@
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170" s="38"/>
+      <c r="A170" s="40"/>
       <c r="B170" s="9" t="s">
         <v>392</v>
       </c>
@@ -7052,7 +7055,7 @@
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" s="39"/>
+      <c r="A171" s="41"/>
       <c r="B171" s="9" t="s">
         <v>394</v>
       </c>
@@ -7061,7 +7064,7 @@
       </c>
     </row>
     <row r="172" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="33" t="s">
+      <c r="A172" s="36" t="s">
         <v>395</v>
       </c>
       <c r="B172" s="1" t="s">
@@ -7072,7 +7075,7 @@
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173" s="36"/>
+      <c r="A173" s="37"/>
       <c r="B173" s="1" t="s">
         <v>399</v>
       </c>
@@ -7081,7 +7084,7 @@
       </c>
     </row>
     <row r="174" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A174" s="36"/>
+      <c r="A174" s="37"/>
       <c r="B174" s="1" t="s">
         <v>401</v>
       </c>
@@ -7090,7 +7093,7 @@
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A175" s="34"/>
+      <c r="A175" s="38"/>
       <c r="B175" s="1" t="s">
         <v>403</v>
       </c>
@@ -7099,7 +7102,7 @@
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176" s="37" t="s">
+      <c r="A176" s="39" t="s">
         <v>404</v>
       </c>
       <c r="B176" s="9" t="s">
@@ -7110,7 +7113,7 @@
       </c>
     </row>
     <row r="177" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A177" s="38"/>
+      <c r="A177" s="40"/>
       <c r="B177" s="9" t="s">
         <v>407</v>
       </c>
@@ -7119,7 +7122,7 @@
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" s="39"/>
+      <c r="A178" s="41"/>
       <c r="B178" s="9" t="s">
         <v>409</v>
       </c>
@@ -7128,7 +7131,7 @@
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" s="33" t="s">
+      <c r="A179" s="36" t="s">
         <v>410</v>
       </c>
       <c r="B179" s="1" t="s">
@@ -7139,7 +7142,7 @@
       </c>
     </row>
     <row r="180" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A180" s="36"/>
+      <c r="A180" s="37"/>
       <c r="B180" s="8" t="s">
         <v>414</v>
       </c>
@@ -7148,7 +7151,7 @@
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181" s="36"/>
+      <c r="A181" s="37"/>
       <c r="B181" s="1" t="s">
         <v>416</v>
       </c>
@@ -7157,7 +7160,7 @@
       </c>
     </row>
     <row r="182" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A182" s="34"/>
+      <c r="A182" s="38"/>
       <c r="B182" s="1" t="s">
         <v>418</v>
       </c>
@@ -7166,7 +7169,7 @@
       </c>
     </row>
     <row r="183" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="37" t="s">
+      <c r="A183" s="39" t="s">
         <v>419</v>
       </c>
       <c r="B183" s="9" t="s">
@@ -7177,7 +7180,7 @@
       </c>
     </row>
     <row r="184" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A184" s="38"/>
+      <c r="A184" s="40"/>
       <c r="B184" s="9" t="s">
         <v>423</v>
       </c>
@@ -7186,7 +7189,7 @@
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185" s="38"/>
+      <c r="A185" s="40"/>
       <c r="B185" s="9" t="s">
         <v>425</v>
       </c>
@@ -7195,7 +7198,7 @@
       </c>
     </row>
     <row r="186" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A186" s="39"/>
+      <c r="A186" s="41"/>
       <c r="B186" s="9" t="s">
         <v>427</v>
       </c>
@@ -7204,7 +7207,7 @@
       </c>
     </row>
     <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A187" s="33" t="s">
+      <c r="A187" s="36" t="s">
         <v>428</v>
       </c>
       <c r="B187" s="1" t="s">
@@ -7215,7 +7218,7 @@
       </c>
     </row>
     <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A188" s="36"/>
+      <c r="A188" s="37"/>
       <c r="B188" s="1" t="s">
         <v>432</v>
       </c>
@@ -7224,7 +7227,7 @@
       </c>
     </row>
     <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A189" s="34"/>
+      <c r="A189" s="38"/>
       <c r="B189" s="1" t="s">
         <v>434</v>
       </c>
@@ -7233,7 +7236,7 @@
       </c>
     </row>
     <row r="190" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="37" t="s">
+      <c r="A190" s="39" t="s">
         <v>435</v>
       </c>
       <c r="B190" s="9" t="s">
@@ -7244,7 +7247,7 @@
       </c>
     </row>
     <row r="191" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A191" s="38"/>
+      <c r="A191" s="40"/>
       <c r="B191" s="9" t="s">
         <v>439</v>
       </c>
@@ -7253,7 +7256,7 @@
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A192" s="39"/>
+      <c r="A192" s="41"/>
       <c r="B192" s="9" t="s">
         <v>441</v>
       </c>
@@ -7262,7 +7265,7 @@
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A193" s="33" t="s">
+      <c r="A193" s="36" t="s">
         <v>442</v>
       </c>
       <c r="B193" s="1" t="s">
@@ -7273,7 +7276,7 @@
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A194" s="36"/>
+      <c r="A194" s="37"/>
       <c r="B194" s="1" t="s">
         <v>446</v>
       </c>
@@ -7282,7 +7285,7 @@
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A195" s="36"/>
+      <c r="A195" s="37"/>
       <c r="B195" s="1" t="s">
         <v>448</v>
       </c>
@@ -7291,7 +7294,7 @@
       </c>
     </row>
     <row r="196" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A196" s="34"/>
+      <c r="A196" s="38"/>
       <c r="B196" s="1" t="s">
         <v>450</v>
       </c>
@@ -7300,7 +7303,7 @@
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A197" s="37" t="s">
+      <c r="A197" s="39" t="s">
         <v>451</v>
       </c>
       <c r="B197" s="9" t="s">
@@ -7311,7 +7314,7 @@
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A198" s="38"/>
+      <c r="A198" s="40"/>
       <c r="B198" s="9" t="s">
         <v>391</v>
       </c>
@@ -7320,7 +7323,7 @@
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A199" s="38"/>
+      <c r="A199" s="40"/>
       <c r="B199" s="9" t="s">
         <v>392</v>
       </c>
@@ -7329,7 +7332,7 @@
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A200" s="38"/>
+      <c r="A200" s="40"/>
       <c r="B200" s="9" t="s">
         <v>456</v>
       </c>
@@ -7338,7 +7341,7 @@
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A201" s="39"/>
+      <c r="A201" s="41"/>
       <c r="B201" s="9" t="s">
         <v>458</v>
       </c>
@@ -7347,7 +7350,7 @@
       </c>
     </row>
     <row r="202" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="33" t="s">
+      <c r="A202" s="36" t="s">
         <v>459</v>
       </c>
       <c r="B202" s="1" t="s">
@@ -7358,7 +7361,7 @@
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A203" s="36"/>
+      <c r="A203" s="37"/>
       <c r="B203" s="1" t="s">
         <v>463</v>
       </c>
@@ -7367,7 +7370,7 @@
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A204" s="36"/>
+      <c r="A204" s="37"/>
       <c r="B204" s="1" t="s">
         <v>465</v>
       </c>
@@ -7376,7 +7379,7 @@
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A205" s="34"/>
+      <c r="A205" s="38"/>
       <c r="B205" s="1" t="s">
         <v>467</v>
       </c>
@@ -7394,7 +7397,7 @@
       <c r="C206" s="23"/>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A207" s="33" t="s">
+      <c r="A207" s="36" t="s">
         <v>469</v>
       </c>
       <c r="B207" s="1" t="s">
@@ -7405,7 +7408,7 @@
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A208" s="36"/>
+      <c r="A208" s="37"/>
       <c r="B208" s="1" t="s">
         <v>472</v>
       </c>
@@ -7414,7 +7417,7 @@
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A209" s="36"/>
+      <c r="A209" s="37"/>
       <c r="B209" s="1" t="s">
         <v>473</v>
       </c>
@@ -7423,7 +7426,7 @@
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A210" s="36"/>
+      <c r="A210" s="37"/>
       <c r="B210" s="1" t="s">
         <v>475</v>
       </c>
@@ -7432,7 +7435,7 @@
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A211" s="36"/>
+      <c r="A211" s="37"/>
       <c r="B211" s="1" t="s">
         <v>476</v>
       </c>
@@ -7441,7 +7444,7 @@
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A212" s="36"/>
+      <c r="A212" s="37"/>
       <c r="B212" s="1" t="s">
         <v>478</v>
       </c>
@@ -7450,7 +7453,7 @@
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A213" s="36"/>
+      <c r="A213" s="37"/>
       <c r="B213" s="1" t="s">
         <v>480</v>
       </c>
@@ -7459,7 +7462,7 @@
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A214" s="34"/>
+      <c r="A214" s="38"/>
       <c r="B214" s="1" t="s">
         <v>481</v>
       </c>
@@ -7468,7 +7471,7 @@
       </c>
     </row>
     <row r="215" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="37" t="s">
+      <c r="A215" s="39" t="s">
         <v>482</v>
       </c>
       <c r="B215" s="9" t="s">
@@ -7479,7 +7482,7 @@
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A216" s="38"/>
+      <c r="A216" s="40"/>
       <c r="B216" s="9" t="s">
         <v>486</v>
       </c>
@@ -7488,7 +7491,7 @@
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A217" s="38"/>
+      <c r="A217" s="40"/>
       <c r="B217" s="9" t="s">
         <v>487</v>
       </c>
@@ -7497,7 +7500,7 @@
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A218" s="39"/>
+      <c r="A218" s="41"/>
       <c r="B218" s="9" t="s">
         <v>488</v>
       </c>
@@ -7506,7 +7509,7 @@
       </c>
     </row>
     <row r="219" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="33" t="s">
+      <c r="A219" s="36" t="s">
         <v>527</v>
       </c>
       <c r="B219" s="1" t="s">
@@ -7517,7 +7520,7 @@
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A220" s="36"/>
+      <c r="A220" s="37"/>
       <c r="B220" s="1" t="s">
         <v>531</v>
       </c>
@@ -7526,7 +7529,7 @@
       </c>
     </row>
     <row r="221" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A221" s="34"/>
+      <c r="A221" s="38"/>
       <c r="B221" s="1" t="s">
         <v>533</v>
       </c>
@@ -7535,7 +7538,7 @@
       </c>
     </row>
     <row r="222" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="37" t="s">
+      <c r="A222" s="39" t="s">
         <v>534</v>
       </c>
       <c r="B222" s="9" t="s">
@@ -7546,7 +7549,7 @@
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A223" s="38"/>
+      <c r="A223" s="40"/>
       <c r="B223" s="9" t="s">
         <v>538</v>
       </c>
@@ -7555,7 +7558,7 @@
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A224" s="38"/>
+      <c r="A224" s="40"/>
       <c r="B224" s="9" t="s">
         <v>540</v>
       </c>
@@ -7564,7 +7567,7 @@
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A225" s="39"/>
+      <c r="A225" s="41"/>
       <c r="B225" s="9" t="s">
         <v>542</v>
       </c>
@@ -7573,7 +7576,7 @@
       </c>
     </row>
     <row r="226" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="33" t="s">
+      <c r="A226" s="36" t="s">
         <v>543</v>
       </c>
       <c r="B226" s="1" t="s">
@@ -7584,7 +7587,7 @@
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A227" s="36"/>
+      <c r="A227" s="37"/>
       <c r="B227" s="1" t="s">
         <v>546</v>
       </c>
@@ -7593,7 +7596,7 @@
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A228" s="34"/>
+      <c r="A228" s="38"/>
       <c r="B228" s="1" t="s">
         <v>548</v>
       </c>
@@ -7602,7 +7605,7 @@
       </c>
     </row>
     <row r="229" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="37" t="s">
+      <c r="A229" s="39" t="s">
         <v>549</v>
       </c>
       <c r="B229" s="9" t="s">
@@ -7613,7 +7616,7 @@
       </c>
     </row>
     <row r="230" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A230" s="38"/>
+      <c r="A230" s="40"/>
       <c r="B230" s="9" t="s">
         <v>553</v>
       </c>
@@ -7622,7 +7625,7 @@
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A231" s="39"/>
+      <c r="A231" s="41"/>
       <c r="B231" s="9" t="s">
         <v>555</v>
       </c>
@@ -7631,7 +7634,7 @@
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A232" s="33" t="s">
+      <c r="A232" s="36" t="s">
         <v>490</v>
       </c>
       <c r="B232" s="1" t="s">
@@ -7642,7 +7645,7 @@
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A233" s="36"/>
+      <c r="A233" s="37"/>
       <c r="B233" s="1" t="s">
         <v>493</v>
       </c>
@@ -7651,7 +7654,7 @@
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A234" s="36"/>
+      <c r="A234" s="37"/>
       <c r="B234" s="1" t="s">
         <v>495</v>
       </c>
@@ -7660,7 +7663,7 @@
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A235" s="34"/>
+      <c r="A235" s="38"/>
       <c r="B235" s="1" t="s">
         <v>497</v>
       </c>
@@ -7680,7 +7683,7 @@
       </c>
     </row>
     <row r="237" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A237" s="33" t="s">
+      <c r="A237" s="36" t="s">
         <v>501</v>
       </c>
       <c r="B237" s="1" t="s">
@@ -7691,7 +7694,7 @@
       </c>
     </row>
     <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A238" s="36"/>
+      <c r="A238" s="37"/>
       <c r="B238" s="1" t="s">
         <v>505</v>
       </c>
@@ -7700,7 +7703,7 @@
       </c>
     </row>
     <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A239" s="34"/>
+      <c r="A239" s="38"/>
       <c r="B239" s="1" t="s">
         <v>507</v>
       </c>
@@ -7709,7 +7712,7 @@
       </c>
     </row>
     <row r="240" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A240" s="37" t="s">
+      <c r="A240" s="39" t="s">
         <v>508</v>
       </c>
       <c r="B240" s="9" t="s">
@@ -7720,7 +7723,7 @@
       </c>
     </row>
     <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A241" s="39"/>
+      <c r="A241" s="41"/>
       <c r="B241" s="9" t="s">
         <v>512</v>
       </c>
@@ -7729,7 +7732,7 @@
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A242" s="33" t="s">
+      <c r="A242" s="36" t="s">
         <v>513</v>
       </c>
       <c r="B242" s="1" t="s">
@@ -7740,7 +7743,7 @@
       </c>
     </row>
     <row r="243" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A243" s="34"/>
+      <c r="A243" s="38"/>
       <c r="B243" s="1" t="s">
         <v>517</v>
       </c>
@@ -7749,7 +7752,7 @@
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A244" s="37" t="s">
+      <c r="A244" s="39" t="s">
         <v>518</v>
       </c>
       <c r="B244" s="9" t="s">
@@ -7760,7 +7763,7 @@
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A245" s="38"/>
+      <c r="A245" s="40"/>
       <c r="B245" s="9" t="s">
         <v>522</v>
       </c>
@@ -7769,7 +7772,7 @@
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A246" s="38"/>
+      <c r="A246" s="40"/>
       <c r="B246" s="9" t="s">
         <v>524</v>
       </c>
@@ -7778,7 +7781,7 @@
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A247" s="39"/>
+      <c r="A247" s="41"/>
       <c r="B247" s="9" t="s">
         <v>526</v>
       </c>
@@ -7787,7 +7790,7 @@
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A248" s="33" t="s">
+      <c r="A248" s="36" t="s">
         <v>556</v>
       </c>
       <c r="B248" s="1" t="s">
@@ -7798,7 +7801,7 @@
       </c>
     </row>
     <row r="249" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A249" s="36"/>
+      <c r="A249" s="37"/>
       <c r="B249" s="1" t="s">
         <v>560</v>
       </c>
@@ -7807,7 +7810,7 @@
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A250" s="34"/>
+      <c r="A250" s="38"/>
       <c r="B250" s="1" t="s">
         <v>562</v>
       </c>
@@ -7816,7 +7819,7 @@
       </c>
     </row>
     <row r="251" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A251" s="37" t="s">
+      <c r="A251" s="39" t="s">
         <v>563</v>
       </c>
       <c r="B251" s="9" t="s">
@@ -7827,7 +7830,7 @@
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A252" s="38"/>
+      <c r="A252" s="40"/>
       <c r="B252" s="9" t="s">
         <v>566</v>
       </c>
@@ -7836,7 +7839,7 @@
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A253" s="38"/>
+      <c r="A253" s="40"/>
       <c r="B253" s="9" t="s">
         <v>568</v>
       </c>
@@ -7845,7 +7848,7 @@
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A254" s="39"/>
+      <c r="A254" s="41"/>
       <c r="B254" s="9" t="s">
         <v>570</v>
       </c>
@@ -7865,7 +7868,7 @@
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A256" s="33" t="s">
+      <c r="A256" s="36" t="s">
         <v>575</v>
       </c>
       <c r="B256" s="1" t="s">
@@ -7876,7 +7879,7 @@
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A257" s="36"/>
+      <c r="A257" s="37"/>
       <c r="B257" s="1" t="s">
         <v>579</v>
       </c>
@@ -7885,7 +7888,7 @@
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A258" s="36"/>
+      <c r="A258" s="37"/>
       <c r="B258" s="1" t="s">
         <v>581</v>
       </c>
@@ -7894,7 +7897,7 @@
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A259" s="34"/>
+      <c r="A259" s="38"/>
       <c r="B259" s="1" t="s">
         <v>583</v>
       </c>
@@ -7903,7 +7906,7 @@
       </c>
     </row>
     <row r="260" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A260" s="33" t="s">
+      <c r="A260" s="36" t="s">
         <v>584</v>
       </c>
       <c r="B260" s="1" t="s">
@@ -7914,7 +7917,7 @@
       </c>
     </row>
     <row r="261" spans="1:3" ht="210" x14ac:dyDescent="0.25">
-      <c r="A261" s="34"/>
+      <c r="A261" s="38"/>
       <c r="B261" s="1" t="s">
         <v>588</v>
       </c>
@@ -8057,7 +8060,7 @@
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A276" s="40" t="s">
+      <c r="A276" s="42" t="s">
         <v>166</v>
       </c>
       <c r="B276" s="1" t="s">
@@ -8068,14 +8071,14 @@
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A277" s="40"/>
+      <c r="A277" s="42"/>
       <c r="B277" s="1" t="s">
         <v>163</v>
       </c>
       <c r="C277" s="1"/>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A278" s="40"/>
+      <c r="A278" s="42"/>
       <c r="B278" s="1" t="s">
         <v>164</v>
       </c>
@@ -8100,7 +8103,7 @@
       <c r="C280" s="1"/>
     </row>
     <row r="281" spans="1:3" ht="180" x14ac:dyDescent="0.25">
-      <c r="A281" s="33" t="s">
+      <c r="A281" s="36" t="s">
         <v>600</v>
       </c>
       <c r="B281" s="1" t="s">
@@ -8111,7 +8114,7 @@
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A282" s="36"/>
+      <c r="A282" s="37"/>
       <c r="B282" s="1" t="s">
         <v>152</v>
       </c>
@@ -8120,14 +8123,14 @@
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A283" s="36"/>
+      <c r="A283" s="37"/>
       <c r="B283" s="1" t="s">
         <v>151</v>
       </c>
       <c r="C283" s="35"/>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A284" s="36"/>
+      <c r="A284" s="37"/>
       <c r="B284" s="1" t="s">
         <v>183</v>
       </c>
@@ -8136,7 +8139,7 @@
       </c>
     </row>
     <row r="285" spans="1:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="A285" s="34"/>
+      <c r="A285" s="38"/>
       <c r="B285" s="1" t="s">
         <v>598</v>
       </c>

</xml_diff>